<commit_message>
Actualizar dashboard Vicuña y Liex
</commit_message>
<xml_diff>
--- a/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
+++ b/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/rigi-dashboard/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0051CB-3E0D-6D4C-8CAA-3236E3CFF468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56A6416-3343-BB45-8BF5-691227B47E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36440" yWindow="0" windowWidth="32360" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="1" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="307">
   <si>
     <t>id_proyecto</t>
   </si>
@@ -438,9 +438,6 @@
     <t>Sal de Vida S.A.</t>
   </si>
   <si>
-    <t>Salterra</t>
-  </si>
-  <si>
     <t>Zijin Mining (LieX S.A.) (China)</t>
   </si>
   <si>
@@ -630,15 +627,6 @@
     <t>Descripción_del_proyecto</t>
   </si>
   <si>
-    <t>desarrollo (factibilidad, permisos) y la construcción de mina, planta e infraestructura asociada para extraer y procesar cátodos de cobre</t>
-  </si>
-  <si>
-    <t>instalación de una planta flotante de licuefacción de gas natural para obtener Gas Natural Licuado (GNL)</t>
-  </si>
-  <si>
-    <t>consiste en la construcción y desarrollo de un oleoducto, Iincrementar la capacidad de transporte y almacenamiento de petróleo crudo viabilizando la exportación de hidrocarburos provenientes de la formación “Vaca Muerta”</t>
-  </si>
-  <si>
     <t>30-70708643-9</t>
   </si>
   <si>
@@ -648,9 +636,6 @@
     <t>Potasio y Litio</t>
   </si>
   <si>
-    <t>extracción directa de litio, nanofiltración y pretratamiento de salmuera que posibilitarán la extracción de litio sin la necesidad de concentración previa en piletas de evaporación, lo que reducirá significativamente el impacto ambiental y la alteración del paisaje, a la vez que también permitirá reducir la generación de residuos y la necesidad de reactivos químicos en el proceso.</t>
-  </si>
-  <si>
     <t>30-69228382-8</t>
   </si>
   <si>
@@ -666,9 +651,6 @@
     <t>Carbonatos Profundos (DCP)</t>
   </si>
   <si>
-    <t>exploración de las concesiones mineras Gualcamayo 1 y Gualcamayo 2 y la determinación de la factibilidad del yacimiento de reservas minerales de oro y plata denominado “Carbonatos Profundos”, y la construcción, puesta en marcha y operación de la planta de tratamiento de dichos minerales extraídos del Proyecto</t>
-  </si>
-  <si>
     <t>Ampliación del Tramo I del Gasoducto Perito Francisco Pascasio Moreno (GPM)</t>
   </si>
   <si>
@@ -684,9 +666,6 @@
     <t>VPU</t>
   </si>
   <si>
-    <t>construcción, financiamiento y Operación y Mantenimiento (O&amp;M) de la infraestructura involucrada para generar una capacidad incremental de catorce millones de metros cúbicos por día (14 MMm³/d) al Tramo I del Gasoducto Francisco Pascasio Moren</t>
-  </si>
-  <si>
     <t>Neuquén; Buenos Aires</t>
   </si>
   <si>
@@ -696,9 +675,6 @@
     <t>30-67305977-1</t>
   </si>
   <si>
-    <t>comprende actividades destinadas a la factibilidad, desarrollo, ejecución y operación del yacimiento de oro y plata “Diablillos”, integrado por quince (15) concesiones mineras contiguas y superpuestas en la zona limítrofe entre las provincias de Salta y Catamarca</t>
-  </si>
-  <si>
     <t>Salta; Catamarca</t>
   </si>
   <si>
@@ -723,9 +699,6 @@
     <t>33-71879284-9</t>
   </si>
   <si>
-    <t>construcción y puesta en operación de una nueva planta de aceros largos, que incluye tanto la acería como la laminadora continua en tándem, de menores emisiones de dióxido de carbono (CO2) respecto de las tecnologías tradicionales y bajo un modelo de producción de economía circular que permitirá reducir el consumo de recursos naturales y disminuir la huella ambiental a partir del uso de un noventa y nueve coma cinco por ciento (99,5%) de chatarra como materia prima</t>
-  </si>
-  <si>
     <t>actividades de industrialización y/o procesamiento del mineral de hierro, el acero y/o sus aleaciones, para la obtención de productos en formas primarias y/o productos elaborados</t>
   </si>
   <si>
@@ -741,12 +714,6 @@
     <t>actividad_subsector_resolución_MECON</t>
   </si>
   <si>
-    <t>construcción de una puerta de enlace multimodal y un punto estratégico de conexión en la Vía Navegable Troncal, también llamada “Hidrovía Paraguay – Paraná”, con el desarrollo de tres (3) unidades de gestión portuaria que buscarán optimizar las operaciones logísticas de carga, descarga, almacenamiento y despacho de distintos tipos de mercaderías, atendiendo a las necesidades de tráfico marítimo y terrestre de la zona </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> instalación de un parque eólico de ciento ochenta (180) megavatios (180 MW) ubicado en la localidad de Olavarría, provincia de Buenos Aires, que también involucra la construcción de una nueva estación transformadora (ET) de treinta y tres a ciento treinta y dos kilovoltios (33/132 Kv) simple barra con dos transformadores de ciento veinte megavoltiamperios (120 MVA) y tres (3) campos, una línea de alta tensión (LAT) de ciento treinta y dos kilovoltios (132 Kv) de aproximadamente veinticinco kilómetros (25 km) de longitud que vinculará el parque eólico con la ET Olavarría -propiedad de TRANSBA SA-, y las obras de ampliación del sistema de transporte que incluirán la repotenciación de los capacitores series en la ET Olavarría y la ampliación de banco de capacitores shunt en la ET Ezeiza</t>
-  </si>
-  <si>
     <t>30-71592816-3</t>
   </si>
   <si>
@@ -756,21 +723,12 @@
     <t>30-71906845-2</t>
   </si>
   <si>
-    <t>construcción de una nueva Planta de Adsorción Selectiva (SA 1B) y una nueva Planta de Carbonato (PC 1B); asimismo, incluye la perforación de pozos de salmuera adicionales, la instalación de estanques, tuberías, servicios públicos y la construcción de edificios auxiliares para apoyar la operación y administración de la nueva producción de carbonato de litio (cf., RE-2025-96020090-APN-SCEYM#MEC), como así también, la construcción de una nueva Planta Compresora de Gas Natural en la localidad de Olacapato, departamento de Los Andes, provincia de Salta, situada dentro del radio de doscientos kilómetros (200 km) del Proyecto, que permitirá ampliar la capacidad de transporte de los gasoductos “La Puna” y “Fénix”, instalaciones asociadas directamente al abastecimiento y transporte de gas natural para la nueva producción del proyecto “Expansión Fase 1B”.</t>
-  </si>
-  <si>
     <t>30-71899846-4</t>
   </si>
   <si>
-    <t>roducción de doce mil (12.000) toneladas anuales de carbonato de litio equivalente (LCE)</t>
-  </si>
-  <si>
     <t>30-71765521-0</t>
   </si>
   <si>
-    <t>parque solar fotovoltaico ubicado en la localidad de Jocolí del departamento Las Heras de la provincia de Mendoza, el cual tendrá una capacidad instalada por un total de trescientos cinco megavatios (305 MW) a desarrollarse en dos (2) etapas y proveerá energía</t>
-  </si>
-  <si>
     <t>Energio Solar</t>
   </si>
   <si>
@@ -907,9 +865,6 @@
   </si>
   <si>
     <t>Gasoducto dedicado para la Exportación de Gas Natural</t>
-  </si>
-  <si>
-    <t>construcción, operación y mantenimiento de un gasoducto dedicado de gas natural destinado exclusivamente a la exportación de Gas Natural Licuado (GNL) que se extenderá desde el Predio Cabecera Tratayén, en la provincia del Neuquén hasta la Estación Compresora San Antonio Oeste en el Golfo San Matías, sito en la provincia de Río Negro, de aproximadamente cuatrocientos ochenta kilómetros (480 km) de longitud, y treinta y seis pulgadas (36”) de diámetro, siendo el objetivo central evacuar la producción incremental de la cuenca Neuquina hacia terminales licuefactoras, aprovechando el potencial de recursos no convencionales provenientes de la formación Vaca Muerta</t>
   </si>
   <si>
     <t> 30-71703621-9</t>
@@ -976,6 +931,90 @@
   </si>
   <si>
     <t>Proyectos de exportación estratégica de largo plazo (PEELP)</t>
+  </si>
+  <si>
+    <t>Res. 1153/2026; Globaris; MECON</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/345075/20260729</t>
+  </si>
+  <si>
+    <t>Res. 1153/2026</t>
+  </si>
+  <si>
+    <t>30-71929244-1</t>
+  </si>
+  <si>
+    <t>Proyecto de la Sucursal Dedicada de Liex S.A.</t>
+  </si>
+  <si>
+    <t>Se identifican signos muy fuertes de preexistencia. El proyecto aprobado bajo RIGI corresponde a LIEX S.A. Sucursal Dedicada en el Salar Tres Quebradas —3Q—, Catamarca. Aunque la Resolución 1153/2026 aprueba una inversión en activos computables por USD 594,136 millones para una planta de 40.000 t/año de carbonato de litio, el proyecto 3Q existía públicamente desde años previos: tuvo evaluación económica preliminar en 2017, estudio de factibilidad en 2021, acuerdo provincial ratificado por ley en 2022, adquisición por Zijin/LIEX en 2022, infraestructura eléctrica asociada tramitada desde 2023–2024 y primera fase en producción desde septiembre de 2025.</t>
+  </si>
+  <si>
+    <t>Construcción y operación de una planta de proceso y de la infraestructura asociada, diseñadas para alcanzar una capacidad de producción de cuarenta mil (40.000) toneladas anuales de carbonato de litio mediante el método de extracción directa</t>
+  </si>
+  <si>
+    <t>Instalación de una planta flotante de licuefacción de gas natural para obtener Gas Natural Licuado (GNL)</t>
+  </si>
+  <si>
+    <t>Consiste en la construcción y desarrollo de un oleoducto, Iincrementar la capacidad de transporte y almacenamiento de petróleo crudo viabilizando la exportación de hidrocarburos provenientes de la formación “Vaca Muerta”</t>
+  </si>
+  <si>
+    <t>Desarrollo (factibilidad, permisos) y la construcción de mina, planta e infraestructura asociada para extraer y procesar cátodos de cobre</t>
+  </si>
+  <si>
+    <t>Extracción directa de litio, nanofiltración y pretratamiento de salmuera que posibilitarán la extracción de litio sin la necesidad de concentración previa en piletas de evaporación, lo que reducirá significativamente el impacto ambiental y la alteración del paisaje, a la vez que también permitirá reducir la generación de residuos y la necesidad de reactivos químicos en el proceso.</t>
+  </si>
+  <si>
+    <t>Exploración de las concesiones mineras Gualcamayo 1 y Gualcamayo 2 y la determinación de la factibilidad del yacimiento de reservas minerales de oro y plata denominado “Carbonatos Profundos”, y la construcción, puesta en marcha y operación de la planta de tratamiento de dichos minerales extraídos del Proyecto</t>
+  </si>
+  <si>
+    <t>Construcción, financiamiento y Operación y Mantenimiento (O&amp;M) de la infraestructura involucrada para generar una capacidad incremental de catorce millones de metros cúbicos por día (14 MMm³/d) al Tramo I del Gasoducto Francisco Pascasio Moren</t>
+  </si>
+  <si>
+    <t>Comprende actividades destinadas a la factibilidad, desarrollo, ejecución y operación del yacimiento de oro y plata “Diablillos”, integrado por quince (15) concesiones mineras contiguas y superpuestas en la zona limítrofe entre las provincias de Salta y Catamarca</t>
+  </si>
+  <si>
+    <t>Construcción y puesta en operación de una nueva planta de aceros largos, que incluye tanto la acería como la laminadora continua en tándem, de menores emisiones de dióxido de carbono (CO2) respecto de las tecnologías tradicionales y bajo un modelo de producción de economía circular que permitirá reducir el consumo de recursos naturales y disminuir la huella ambiental a partir del uso de un noventa y nueve coma cinco por ciento (99,5%) de chatarra como materia prima</t>
+  </si>
+  <si>
+    <t>Construcción de una puerta de enlace multimodal y un punto estratégico de conexión en la Vía Navegable Troncal, también llamada “Hidrovía Paraguay – Paraná”, con el desarrollo de tres (3) unidades de gestión portuaria que buscarán optimizar las operaciones logísticas de carga, descarga, almacenamiento y despacho de distintos tipos de mercaderías, atendiendo a las necesidades de tráfico marítimo y terrestre de la zona </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Instalación de un parque eólico de ciento ochenta (180) megavatios (180 MW) ubicado en la localidad de Olavarría, provincia de Buenos Aires, que también involucra la construcción de una nueva estación transformadora (ET) de treinta y tres a ciento treinta y dos kilovoltios (33/132 Kv) simple barra con dos transformadores de ciento veinte megavoltiamperios (120 MVA) y tres (3) campos, una línea de alta tensión (LAT) de ciento treinta y dos kilovoltios (132 Kv) de aproximadamente veinticinco kilómetros (25 km) de longitud que vinculará el parque eólico con la ET Olavarría -propiedad de TRANSBA SA-, y las obras de ampliación del sistema de transporte que incluirán la repotenciación de los capacitores series en la ET Olavarría y la ampliación de banco de capacitores shunt en la ET Ezeiza</t>
+  </si>
+  <si>
+    <t>Construcción de una nueva Planta de Adsorción Selectiva (SA 1B) y una nueva Planta de Carbonato (PC 1B); asimismo, incluye la perforación de pozos de salmuera adicionales, la instalación de estanques, tuberías, servicios públicos y la construcción de edificios auxiliares para apoyar la operación y administración de la nueva producción de carbonato de litio (cf., RE-2025-96020090-APN-SCEYM#MEC), como así también, la construcción de una nueva Planta Compresora de Gas Natural en la localidad de Olacapato, departamento de Los Andes, provincia de Salta, situada dentro del radio de doscientos kilómetros (200 km) del Proyecto, que permitirá ampliar la capacidad de transporte de los gasoductos “La Puna” y “Fénix”, instalaciones asociadas directamente al abastecimiento y transporte de gas natural para la nueva producción del proyecto “Expansión Fase 1B”.</t>
+  </si>
+  <si>
+    <t>Producción de doce mil (12.000) toneladas anuales de carbonato de litio equivalente (LCE)</t>
+  </si>
+  <si>
+    <t>Parque solar fotovoltaico ubicado en la localidad de Jocolí del departamento Las Heras de la provincia de Mendoza, el cual tendrá una capacidad instalada por un total de trescientos cinco megavatios (305 MW) a desarrollarse en dos (2) etapas y proveerá energía</t>
+  </si>
+  <si>
+    <t>Construcción, operación y mantenimiento de un gasoducto dedicado de gas natural destinado exclusivamente a la exportación de Gas Natural Licuado (GNL) que se extenderá desde el Predio Cabecera Tratayén, en la provincia del Neuquén hasta la Estación Compresora San Antonio Oeste en el Golfo San Matías, sito en la provincia de Río Negro, de aproximadamente cuatrocientos ochenta kilómetros (480 km) de longitud, y treinta y seis pulgadas (36”) de diámetro, siendo el objetivo central evacuar la producción incremental de la cuenca Neuquina hacia terminales licuefactoras, aprovechando el potencial de recursos no convencionales provenientes de la formación Vaca Muerta</t>
+  </si>
+  <si>
+    <t>33-61913055-9</t>
+  </si>
+  <si>
+    <t>Extracción, producción y exportación de cobre, oro y plata de los yacimientos Josemaría y Filo del Sol ubicados en la provincia de San Juan, República Argentina, así como la exploración de las concesiones mineras que forman parte del proyecto y el desarrollo de la infraestructura necesaria para su ejecución.</t>
+  </si>
+  <si>
+    <t>Cobre, Oro y Plata</t>
+  </si>
+  <si>
+    <t>Res. 1154/2026</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/345167/20260730</t>
+  </si>
+  <si>
+    <t>Res. 1154/2026; Globaris; MECON</t>
+  </si>
+  <si>
+    <t>Antes del anuncio inicial del RIGI, Josemaría ya contaba con una factibilidad de noviembre de 2020, una evaluación ambiental aprobada en abril de 2022, ingeniería, adquisición de equipos de larga entrega y USD 276 millones de gastos de capital durante 2023; Filo del Sol también poseía prefactibilidades y exploración avanzada. Estos antecedentes corresponden a los mismos depósitos y, principalmente, a la actual primera etapa basada en Josemaría. Sin embargo, la sociedad conjunta BHP–Lundin se constituyó en enero de 2025, la primera evaluación técnica unificada apareció en febrero de 2026 y la decisión final de inversión continuaba pendiente después de la aprobación.</t>
   </si>
 </sst>
 </file>
@@ -1125,7 +1164,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1174,10 +1213,7 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1187,6 +1223,20 @@
     <cellStyle name="Notas" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="27">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1595,20 +1645,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
@@ -1640,32 +1676,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProyectosIntegrados" displayName="ProyectosIntegrados" ref="A1:X40" headerRowDxfId="26" dataDxfId="25" totalsRowDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProyectosIntegrados" displayName="ProyectosIntegrados" ref="A1:X40" headerRowDxfId="26" dataDxfId="0" totalsRowDxfId="25">
   <tableColumns count="24">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="VPU" dataDxfId="23"/>
-    <tableColumn id="22" xr3:uid="{48F4E9CA-8EE4-9B46-B775-30029B62248E}" name="Descripción_del_proyecto" dataDxfId="22"/>
-    <tableColumn id="19" xr3:uid="{59A3C3BF-E3A1-3748-85BC-5ADA196D8039}" name="Proyectos de exportación estratégica de largo plazo (PEELP)" dataDxfId="21"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="id_proyecto" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="empresa" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="titular_proyecto" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{E1C7B229-46A1-4B4F-9ADD-A9E811939D67}" name="CUIT" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="sector" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="subsector" dataDxfId="15"/>
-    <tableColumn id="18" xr3:uid="{3AFF64F9-973D-4A41-865B-D4166A5841A1}" name="actividad_subsector_resolución_MECON" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="provincia" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="localidad_region" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Monto (mill. USD)" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Activos Computables (mill. USD)" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Estado administrativo" dataDxfId="9"/>
-    <tableColumn id="24" xr3:uid="{00D6C894-3563-A741-A5B5-7FF8DB602F8A}" name="Empleos (directos e indirectos)" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="fecha_presentacion" dataDxfId="7"/>
-    <tableColumn id="21" xr3:uid="{D27A2121-7D63-544C-B031-C3DB1A1B8B6A}" name="fecha_adhesion_rigi" dataDxfId="6"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="fecha_publicacion_bo" dataDxfId="5"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="norma_aprobacion" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{B0966B39-0FA3-9146-96DB-BD345771FAC8}" name="Clasificacion_preexistencia_boletin_oficial" dataDxfId="3"/>
-    <tableColumn id="23" xr3:uid="{36F41A70-CDCD-0440-8E79-C4973DF4F4B3}" name="Justificacion_preexistencia_boletin_oficial" dataDxfId="2"/>
-    <tableColumn id="16" xr3:uid="{BC53B1FB-4807-D244-BE0E-F220BF050122}" name="link_norma" dataDxfId="1"/>
-    <tableColumn id="20" xr3:uid="{6C16FCDF-822E-B843-A888-4F4B69680144}" name="Fuentes" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="VPU" dataDxfId="24"/>
+    <tableColumn id="22" xr3:uid="{48F4E9CA-8EE4-9B46-B775-30029B62248E}" name="Descripción_del_proyecto" dataDxfId="23"/>
+    <tableColumn id="19" xr3:uid="{59A3C3BF-E3A1-3748-85BC-5ADA196D8039}" name="Proyectos de exportación estratégica de largo plazo (PEELP)" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="id_proyecto" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="empresa" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="titular_proyecto" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{E1C7B229-46A1-4B4F-9ADD-A9E811939D67}" name="CUIT" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="sector" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="subsector" dataDxfId="16"/>
+    <tableColumn id="18" xr3:uid="{3AFF64F9-973D-4A41-865B-D4166A5841A1}" name="actividad_subsector_resolución_MECON" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="provincia" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="localidad_region" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Monto (mill. USD)" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Activos Computables (mill. USD)" dataDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Estado administrativo" dataDxfId="10"/>
+    <tableColumn id="24" xr3:uid="{00D6C894-3563-A741-A5B5-7FF8DB602F8A}" name="Empleos (directos e indirectos)" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="fecha_presentacion" dataDxfId="8"/>
+    <tableColumn id="21" xr3:uid="{D27A2121-7D63-544C-B031-C3DB1A1B8B6A}" name="fecha_adhesion_rigi" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="fecha_publicacion_bo" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="norma_aprobacion" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{B0966B39-0FA3-9146-96DB-BD345771FAC8}" name="Clasificacion_preexistencia_boletin_oficial" dataDxfId="4"/>
+    <tableColumn id="23" xr3:uid="{36F41A70-CDCD-0440-8E79-C4973DF4F4B3}" name="Justificacion_preexistencia_boletin_oficial" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{BC53B1FB-4807-D244-BE0E-F220BF050122}" name="link_norma" dataDxfId="2"/>
+    <tableColumn id="20" xr3:uid="{6C16FCDF-822E-B843-A888-4F4B69680144}" name="Fuentes" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1872,13 +1908,13 @@
   <sheetData>
     <row r="1" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
@@ -1887,10 +1923,10 @@
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>2</v>
@@ -1899,7 +1935,7 @@
         <v>3</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>4</v>
@@ -1908,40 +1944,40 @@
         <v>5</v>
       </c>
       <c r="M1" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="N1" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="O1" s="4" t="s">
-        <v>149</v>
-      </c>
       <c r="P1" s="4" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="Q1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="R1" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="S1" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>179</v>
       </c>
       <c r="T1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="W1" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="X1" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="30" x14ac:dyDescent="0.15">
@@ -1949,10 +1985,10 @@
         <v>40</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>186</v>
+        <v>286</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D2" s="8">
         <v>7</v>
@@ -1961,19 +1997,19 @@
         <v>41</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G2" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>168</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>169</v>
       </c>
       <c r="K2" s="7" t="s">
         <v>42</v>
@@ -2006,27 +2042,27 @@
         <v>43</v>
       </c>
       <c r="U2" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V2" s="7" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="W2" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="X2" s="7" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" spans="1:24" ht="45" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>187</v>
+        <v>287</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D3" s="8">
         <v>13</v>
@@ -2038,16 +2074,16 @@
         <v>67</v>
       </c>
       <c r="G3" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="J3" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>175</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>42</v>
@@ -2080,27 +2116,27 @@
         <v>68</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V3" s="7" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="W3" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="X3" s="7" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="45" x14ac:dyDescent="0.15">
       <c r="A4" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>185</v>
+        <v>288</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D4" s="8">
         <v>33</v>
@@ -2112,7 +2148,7 @@
         <v>76</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>19</v>
@@ -2121,7 +2157,7 @@
         <v>52</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>25</v>
@@ -2154,27 +2190,27 @@
         <v>77</v>
       </c>
       <c r="U4" s="7" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="V4" s="7" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="X4" s="7" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="60" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>191</v>
+        <v>289</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D5" s="8">
         <v>10</v>
@@ -2186,7 +2222,7 @@
         <v>55</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>19</v>
@@ -2195,7 +2231,7 @@
         <v>56</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>20</v>
@@ -2228,16 +2264,16 @@
         <v>57</v>
       </c>
       <c r="U5" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V5" s="7" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="W5" s="12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="X5" s="7" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="45" x14ac:dyDescent="0.15">
@@ -2245,10 +2281,10 @@
         <v>49</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D6" s="8">
         <v>9</v>
@@ -2260,7 +2296,7 @@
         <v>51</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>19</v>
@@ -2269,7 +2305,7 @@
         <v>52</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>38</v>
@@ -2302,27 +2338,27 @@
         <v>53</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V6" s="7" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="W6" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="X6" s="7" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="45" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>197</v>
+        <v>290</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D7" s="8">
         <v>3</v>
@@ -2334,16 +2370,16 @@
         <v>24</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>25</v>
@@ -2376,27 +2412,27 @@
         <v>27</v>
       </c>
       <c r="U7" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V7" s="13" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
       <c r="W7" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="X7" s="7" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="45" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>203</v>
+        <v>291</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D8" s="8">
         <v>1</v>
@@ -2408,22 +2444,22 @@
         <v>9</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="M8" s="9">
         <v>550</v>
@@ -2450,16 +2486,16 @@
         <v>13</v>
       </c>
       <c r="U8" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V8" s="7" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="W8" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="X8" s="7" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="45" x14ac:dyDescent="0.15">
@@ -2467,10 +2503,10 @@
         <v>16</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>207</v>
+        <v>292</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D9" s="8">
         <v>2</v>
@@ -2482,19 +2518,19 @@
         <v>18</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>21</v>
@@ -2524,27 +2560,27 @@
         <v>22</v>
       </c>
       <c r="U9" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V9" s="7" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="W9" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="X9" s="7" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="75" x14ac:dyDescent="0.15">
       <c r="A10" s="14" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D10" s="8">
         <v>14</v>
@@ -2553,19 +2589,19 @@
         <v>69</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>25</v>
@@ -2598,16 +2634,16 @@
         <v>70</v>
       </c>
       <c r="U10" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V10" s="7" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
       <c r="W10" s="15" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="X10" s="7" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="75" x14ac:dyDescent="0.15">
@@ -2615,10 +2651,10 @@
         <v>44</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>216</v>
+        <v>293</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D11" s="8">
         <v>8</v>
@@ -2630,7 +2666,7 @@
         <v>46</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>47</v>
@@ -2639,7 +2675,7 @@
         <v>47</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>32</v>
@@ -2672,27 +2708,27 @@
         <v>48</v>
       </c>
       <c r="U11" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V11" s="7" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="W11" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="X11" s="7" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="60" x14ac:dyDescent="0.15">
       <c r="A12" s="7" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>222</v>
+        <v>294</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D12" s="8">
         <v>12</v>
@@ -2704,7 +2740,7 @@
         <v>61</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>62</v>
@@ -2713,7 +2749,7 @@
         <v>63</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>64</v>
@@ -2746,16 +2782,16 @@
         <v>65</v>
       </c>
       <c r="U12" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V12" s="7" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="W12" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="X12" s="7" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="120" x14ac:dyDescent="0.15">
@@ -2763,10 +2799,10 @@
         <v>28</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>223</v>
+        <v>295</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D13" s="8">
         <v>4</v>
@@ -2778,7 +2814,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>10</v>
@@ -2820,27 +2856,27 @@
         <v>34</v>
       </c>
       <c r="U13" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V13" s="7" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="W13" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="X13" s="7" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="120" x14ac:dyDescent="0.15">
       <c r="A14" s="7" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>227</v>
+        <v>296</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D14" s="8">
         <v>11</v>
@@ -2849,10 +2885,10 @@
         <v>54</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>19</v>
@@ -2861,7 +2897,7 @@
         <v>56</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>58</v>
@@ -2894,16 +2930,16 @@
         <v>59</v>
       </c>
       <c r="U14" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V14" s="7" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="W14" s="12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="X14" s="7" t="s">
-        <v>273</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="45" x14ac:dyDescent="0.15">
@@ -2911,10 +2947,10 @@
         <v>71</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>229</v>
+        <v>297</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D15" s="8">
         <v>39</v>
@@ -2926,7 +2962,7 @@
         <v>73</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>19</v>
@@ -2935,7 +2971,7 @@
         <v>56</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>58</v>
@@ -2968,16 +3004,16 @@
         <v>74</v>
       </c>
       <c r="U15" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V15" s="7" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="W15" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="45" x14ac:dyDescent="0.15">
@@ -2985,10 +3021,10 @@
         <v>35</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>231</v>
+        <v>298</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D16" s="8">
         <v>5</v>
@@ -3000,13 +3036,13 @@
         <v>37</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>230</v>
+        <v>217</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="J16" s="7"/>
       <c r="K16" s="7" t="s">
@@ -3040,16 +3076,16 @@
         <v>39</v>
       </c>
       <c r="U16" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V16" s="13" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="W16" s="12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="X16" s="7" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3086,7 +3122,7 @@
       </c>
       <c r="N17" s="9"/>
       <c r="O17" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P17" s="7"/>
       <c r="Q17" s="10">
@@ -3099,7 +3135,7 @@
       <c r="V17" s="7"/>
       <c r="W17" s="12"/>
       <c r="X17" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3136,7 +3172,7 @@
       </c>
       <c r="N18" s="9"/>
       <c r="O18" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P18" s="7"/>
       <c r="Q18" s="10">
@@ -3149,7 +3185,7 @@
       <c r="V18" s="7"/>
       <c r="W18" s="15"/>
       <c r="X18" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3186,7 +3222,7 @@
       </c>
       <c r="N19" s="9"/>
       <c r="O19" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P19" s="7"/>
       <c r="Q19" s="10">
@@ -3199,18 +3235,18 @@
       <c r="V19" s="7"/>
       <c r="W19" s="15"/>
       <c r="X19" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="20" spans="1:24" ht="45" x14ac:dyDescent="0.15">
       <c r="A20" s="7" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D20" s="8">
         <v>18</v>
@@ -3219,10 +3255,10 @@
         <v>90</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>19</v>
@@ -3231,7 +3267,7 @@
         <v>56</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>91</v>
@@ -3261,19 +3297,19 @@
         <v>46177</v>
       </c>
       <c r="T20" s="7" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
       <c r="U20" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V20" s="7" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="W20" s="15" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
       <c r="X20" s="7" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3310,7 +3346,7 @@
       </c>
       <c r="N21" s="9"/>
       <c r="O21" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P21" s="7"/>
       <c r="Q21" s="10">
@@ -3323,7 +3359,7 @@
       <c r="V21" s="7"/>
       <c r="W21" s="15"/>
       <c r="X21" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3360,7 +3396,7 @@
       </c>
       <c r="N22" s="9"/>
       <c r="O22" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P22" s="7"/>
       <c r="Q22" s="10">
@@ -3373,7 +3409,7 @@
       <c r="V22" s="7"/>
       <c r="W22" s="15"/>
       <c r="X22" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3410,7 +3446,7 @@
       </c>
       <c r="N23" s="9"/>
       <c r="O23" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P23" s="7"/>
       <c r="Q23" s="10">
@@ -3423,12 +3459,12 @@
       <c r="V23" s="7"/>
       <c r="W23" s="15"/>
       <c r="X23" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A24" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="7"/>
@@ -3439,7 +3475,7 @@
         <v>114</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G24" s="14"/>
       <c r="H24" s="9" t="s">
@@ -3460,7 +3496,7 @@
       </c>
       <c r="N24" s="9"/>
       <c r="O24" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P24" s="7"/>
       <c r="Q24" s="10">
@@ -3473,42 +3509,42 @@
       <c r="V24" s="7"/>
       <c r="W24" s="15"/>
       <c r="X24" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="90" x14ac:dyDescent="0.15">
       <c r="A25" s="7" t="s">
-        <v>277</v>
+        <v>263</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>278</v>
+        <v>299</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D25" s="8">
         <v>38</v>
       </c>
       <c r="E25" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F25" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>140</v>
-      </c>
       <c r="G25" s="7" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="L25" s="7" t="s">
         <v>12</v>
@@ -3535,24 +3571,24 @@
         <v>46198</v>
       </c>
       <c r="T25" s="7" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="U25" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V25" s="7" t="s">
-        <v>284</v>
+        <v>269</v>
       </c>
       <c r="W25" s="12" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="X25" s="7" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
     </row>
     <row r="26" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A26" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -3560,10 +3596,10 @@
         <v>40</v>
       </c>
       <c r="E26" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="F26" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="G26" s="7"/>
       <c r="H26" s="9" t="s">
@@ -3584,7 +3620,7 @@
       </c>
       <c r="N26" s="9"/>
       <c r="O26" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P26" s="7"/>
       <c r="Q26" s="10">
@@ -3597,12 +3633,12 @@
       <c r="V26" s="7"/>
       <c r="W26" s="7"/>
       <c r="X26" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A27" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -3610,7 +3646,7 @@
         <v>41</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>14</v>
@@ -3634,7 +3670,7 @@
       </c>
       <c r="N27" s="9"/>
       <c r="O27" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P27" s="7"/>
       <c r="Q27" s="10">
@@ -3647,12 +3683,12 @@
       <c r="V27" s="7"/>
       <c r="W27" s="7"/>
       <c r="X27" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="28" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A28" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -3660,7 +3696,7 @@
         <v>32</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>14</v>
@@ -3684,7 +3720,7 @@
       </c>
       <c r="N28" s="9"/>
       <c r="O28" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P28" s="7"/>
       <c r="Q28" s="10">
@@ -3697,12 +3733,12 @@
       <c r="V28" s="7"/>
       <c r="W28" s="7"/>
       <c r="X28" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="29" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A29" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="7"/>
@@ -3710,10 +3746,10 @@
         <v>34</v>
       </c>
       <c r="E29" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F29" s="14" t="s">
         <v>130</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>131</v>
       </c>
       <c r="G29" s="14"/>
       <c r="H29" s="9" t="s">
@@ -3734,7 +3770,7 @@
       </c>
       <c r="N29" s="9"/>
       <c r="O29" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P29" s="7"/>
       <c r="Q29" s="10">
@@ -3747,12 +3783,12 @@
       <c r="V29" s="7"/>
       <c r="W29" s="7"/>
       <c r="X29" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="30" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A30" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -3760,10 +3796,10 @@
         <v>35</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G30" s="7"/>
       <c r="H30" s="9" t="s">
@@ -3784,7 +3820,7 @@
       </c>
       <c r="N30" s="9"/>
       <c r="O30" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P30" s="7"/>
       <c r="Q30" s="10">
@@ -3797,12 +3833,12 @@
       <c r="V30" s="7"/>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="15" x14ac:dyDescent="0.15">
       <c r="A31" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -3813,7 +3849,7 @@
         <v>96</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G31" s="7"/>
       <c r="H31" s="9" t="s">
@@ -3834,7 +3870,7 @@
       </c>
       <c r="N31" s="9"/>
       <c r="O31" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P31" s="7"/>
       <c r="Q31" s="10">
@@ -3847,7 +3883,7 @@
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
       <c r="X31" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="32" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3884,7 +3920,7 @@
       </c>
       <c r="N32" s="9"/>
       <c r="O32" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P32" s="7"/>
       <c r="Q32" s="10" t="s">
@@ -3897,7 +3933,7 @@
       <c r="V32" s="7"/>
       <c r="W32" s="7"/>
       <c r="X32" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3934,7 +3970,7 @@
       </c>
       <c r="N33" s="9"/>
       <c r="O33" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P33" s="7"/>
       <c r="Q33" s="10">
@@ -3947,7 +3983,7 @@
       <c r="V33" s="7"/>
       <c r="W33" s="7"/>
       <c r="X33" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="34" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -3984,7 +4020,7 @@
       </c>
       <c r="N34" s="9"/>
       <c r="O34" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P34" s="7"/>
       <c r="Q34" s="10">
@@ -3997,7 +4033,7 @@
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
       <c r="X34" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -4034,7 +4070,7 @@
       </c>
       <c r="N35" s="9"/>
       <c r="O35" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P35" s="7"/>
       <c r="Q35" s="10">
@@ -4047,18 +4083,18 @@
       <c r="V35" s="7"/>
       <c r="W35" s="7"/>
       <c r="X35" s="7" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="36" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" ht="90" x14ac:dyDescent="0.15">
       <c r="A36" s="7" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>291</v>
+        <v>276</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D36" s="8">
         <v>26</v>
@@ -4070,16 +4106,16 @@
         <v>115</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>290</v>
+        <v>275</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J36" s="17" t="s">
-        <v>289</v>
+        <v>274</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>89</v>
@@ -4109,19 +4145,19 @@
         <v>46224</v>
       </c>
       <c r="T36" s="7" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="V36" s="18" t="s">
-        <v>292</v>
+        <v>169</v>
+      </c>
+      <c r="V36" s="16" t="s">
+        <v>277</v>
       </c>
       <c r="W36" s="7" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="X36" s="7" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -4158,7 +4194,7 @@
       </c>
       <c r="N37" s="9"/>
       <c r="O37" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P37" s="7"/>
       <c r="Q37" s="10">
@@ -4171,7 +4207,7 @@
       <c r="V37" s="7"/>
       <c r="W37" s="7"/>
       <c r="X37" s="7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="38" spans="1:24" ht="15" x14ac:dyDescent="0.15">
@@ -4208,7 +4244,7 @@
       </c>
       <c r="N38" s="9"/>
       <c r="O38" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P38" s="7"/>
       <c r="Q38" s="10">
@@ -4221,32 +4257,38 @@
       <c r="V38" s="7"/>
       <c r="W38" s="7"/>
       <c r="X38" s="7" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="39" spans="1:24" ht="15" x14ac:dyDescent="0.15">
-      <c r="A39" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="B39" s="7"/>
+        <v>226</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" ht="90" x14ac:dyDescent="0.15">
+      <c r="A39" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>285</v>
+      </c>
       <c r="C39" s="7"/>
       <c r="D39" s="8">
         <v>29</v>
       </c>
       <c r="E39" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F39" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="G39" s="7"/>
+      <c r="G39" s="17" t="s">
+        <v>282</v>
+      </c>
       <c r="H39" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I39" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J39" s="7"/>
+      <c r="J39" s="7" t="s">
+        <v>186</v>
+      </c>
       <c r="K39" s="7" t="s">
         <v>58</v>
       </c>
@@ -4256,47 +4298,71 @@
       <c r="M39" s="9">
         <v>710</v>
       </c>
-      <c r="N39" s="9"/>
+      <c r="N39" s="9">
+        <v>594.13599999999997</v>
+      </c>
       <c r="O39" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="P39" s="7"/>
-      <c r="Q39" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="R39" s="10"/>
-      <c r="S39" s="10"/>
-      <c r="T39" s="7"/>
-      <c r="U39" s="7"/>
-      <c r="V39" s="7"/>
-      <c r="W39" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="P39" s="7">
+        <v>4406</v>
+      </c>
+      <c r="Q39" s="10">
+        <v>46063</v>
+      </c>
+      <c r="R39" s="10">
+        <v>46206</v>
+      </c>
+      <c r="S39" s="10">
+        <v>46232</v>
+      </c>
+      <c r="T39" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="V39" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="W39" s="7" t="s">
+        <v>280</v>
+      </c>
       <c r="X39" s="7" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="40" spans="1:24" ht="15" x14ac:dyDescent="0.15">
-      <c r="A40" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="B40" s="7"/>
-      <c r="C40" s="7"/>
+        <v>279</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" ht="90" x14ac:dyDescent="0.15">
+      <c r="A40" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>169</v>
+      </c>
       <c r="D40" s="8">
         <v>31</v>
       </c>
       <c r="E40" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F40" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="F40" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="G40" s="7"/>
+      <c r="G40" s="17" t="s">
+        <v>300</v>
+      </c>
       <c r="H40" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="J40" s="7"/>
+        <v>302</v>
+      </c>
+      <c r="J40" s="14" t="s">
+        <v>179</v>
+      </c>
       <c r="K40" s="7" t="s">
         <v>25</v>
       </c>
@@ -4304,24 +4370,40 @@
         <v>26</v>
       </c>
       <c r="M40" s="9">
-        <v>9712</v>
-      </c>
-      <c r="N40" s="9"/>
+        <v>9737.0139999999992</v>
+      </c>
+      <c r="N40" s="9">
+        <v>9024.7322810000005</v>
+      </c>
       <c r="O40" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="P40" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="P40" s="7">
+        <v>30000</v>
+      </c>
       <c r="Q40" s="10">
         <v>46002</v>
       </c>
-      <c r="R40" s="10"/>
-      <c r="S40" s="10"/>
-      <c r="T40" s="7"/>
-      <c r="U40" s="7"/>
-      <c r="V40" s="7"/>
-      <c r="W40" s="7"/>
+      <c r="R40" s="10">
+        <v>46176</v>
+      </c>
+      <c r="S40" s="10">
+        <v>46233</v>
+      </c>
+      <c r="T40" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="U40" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="V40" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="W40" s="15" t="s">
+        <v>304</v>
+      </c>
       <c r="X40" s="7" t="s">
-        <v>240</v>
+        <v>305</v>
       </c>
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.15">
@@ -4577,11 +4659,12 @@
     <hyperlink ref="W14" r:id="rId14" xr:uid="{56EA8146-7375-2940-8CE7-621D3D82E155}"/>
     <hyperlink ref="W15" r:id="rId15" xr:uid="{B991F48F-963A-5548-9E1D-97F06C683698}"/>
     <hyperlink ref="W20" r:id="rId16" xr:uid="{AE74A4E6-305E-5F49-B0FE-9AAB97F6A3DF}"/>
+    <hyperlink ref="W40" r:id="rId17" xr:uid="{58E4C55D-2972-6044-88B9-E8D053273528}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId17"/>
+  <legacyDrawing r:id="rId18"/>
   <tableParts count="1">
-    <tablePart r:id="rId18"/>
+    <tablePart r:id="rId19"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4596,7 +4679,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualización 30 julio 2026
</commit_message>
<xml_diff>
--- a/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
+++ b/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56A6416-3343-BB45-8BF5-691227B47E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B70C9F-C055-7A4F-93F9-A7FEFFAD449A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36440" yWindow="0" windowWidth="32360" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,12 +36,14 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={DBA8E842-1B69-4E44-955F-86A6656A5A38}</author>
-    <author>tc={2603CD78-4DA2-7245-9496-2BEE29538FD4}</author>
-    <author>tc={D89771A4-99A8-0740-A054-82109EE9B8C1}</author>
+    <author>tc={CC7FC192-DD2F-524F-965B-B519233399BD}</author>
+    <author>tc={EA61046C-C94E-C449-8761-ABD505A37332}</author>
+    <author>tc={9E845984-16BC-D640-8568-DCBC39BD282B}</author>
+    <author>tc={D756854B-3370-2C47-8E59-D458EBCA5109}</author>
+    <author>tc={909B81E5-AB38-BB4F-A77E-C63D2711848A}</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{DBA8E842-1B69-4E44-955F-86A6656A5A38}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{CC7FC192-DD2F-524F-965B-B519233399BD}">
       <text>
         <t xml:space="preserve">[Comentario encadenado]
 Tu versión de Excel te permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -50,7 +52,24 @@
 </t>
       </text>
     </comment>
-    <comment ref="P1" authorId="1" shapeId="0" xr:uid="{2603CD78-4DA2-7245-9496-2BEE29538FD4}">
+    <comment ref="M1" authorId="1" shapeId="0" xr:uid="{EA61046C-C94E-C449-8761-ABD505A37332}">
+      <text>
+        <t xml:space="preserve">[Comentario encadenado]
+Tu versión de Excel te permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    En los casos en que el monto total de inversión informado en el sitio web oficial del RIGI difiere del consignado en la resolución correspondiente a cada proyecto aprobado, se utiliza el monto publicado en el sitio web oficial del régimen.
+</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="2" shapeId="0" xr:uid="{9E845984-16BC-D640-8568-DCBC39BD282B}">
+      <text>
+        <t>[Comentario encadenado]
+Tu versión de Excel te permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Se completo los datos de inversión total de los proyectos aprobados con los montos reportados en la resolución respectiva de cada proyecto. En algunos casos los montos reportados difieren en comparación a los reportados en el sitio web oficial del RIGI del gobierno</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="3" shapeId="0" xr:uid="{D756854B-3370-2C47-8E59-D458EBCA5109}">
       <text>
         <t xml:space="preserve">[Comentario encadenado]
 Tu versión de Excel te permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -59,7 +78,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="M3" authorId="2" shapeId="0" xr:uid="{D89771A4-99A8-0740-A054-82109EE9B8C1}">
+    <comment ref="N3" authorId="4" shapeId="0" xr:uid="{909B81E5-AB38-BB4F-A77E-C63D2711848A}">
       <text>
         <t xml:space="preserve">[Comentario encadenado]
 Tu versión de Excel te permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -73,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="309">
   <si>
     <t>id_proyecto</t>
   </si>
@@ -915,9 +934,6 @@
     <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/344628/20260721</t>
   </si>
   <si>
-    <t>Res. 1015/2026</t>
-  </si>
-  <si>
     <t>Explotación y Producción de Hidrocarburos Líquidos y Gaseosos Costa Adentro</t>
   </si>
   <si>
@@ -999,9 +1015,6 @@
     <t>33-61913055-9</t>
   </si>
   <si>
-    <t>Extracción, producción y exportación de cobre, oro y plata de los yacimientos Josemaría y Filo del Sol ubicados en la provincia de San Juan, República Argentina, así como la exploración de las concesiones mineras que forman parte del proyecto y el desarrollo de la infraestructura necesaria para su ejecución.</t>
-  </si>
-  <si>
     <t>Cobre, Oro y Plata</t>
   </si>
   <si>
@@ -1015,6 +1028,18 @@
   </si>
   <si>
     <t>Antes del anuncio inicial del RIGI, Josemaría ya contaba con una factibilidad de noviembre de 2020, una evaluación ambiental aprobada en abril de 2022, ingeniería, adquisición de equipos de larga entrega y USD 276 millones de gastos de capital durante 2023; Filo del Sol también poseía prefactibilidades y exploración avanzada. Estos antecedentes corresponden a los mismos depósitos y, principalmente, a la actual primera etapa basada en Josemaría. Sin embargo, la sociedad conjunta BHP–Lundin se constituyó en enero de 2025, la primera evaluación técnica unificada apareció en febrero de 2026 y la decisión final de inversión continuaba pendiente después de la aprobación.</t>
+  </si>
+  <si>
+    <t>Monto (mill. USD) - aprobados resolución</t>
+  </si>
+  <si>
+    <t>Expansión Fase 1B</t>
+  </si>
+  <si>
+    <t>Res. 1025/2026</t>
+  </si>
+  <si>
+    <t>Extracción, producción y exportación de cobre, oro y plata de los yacimientos Josemaría y Filo del Sol ubicados en la provincia de San Juan, República Argentina, así como la exploración de las concesiones mineras que forman parte del proyecto y el desarrollo de la infraestructura necesaria para su ejecución. Incluye infraestructura clave para operaciones de minería a cielo abierto: una planta concentradora para el procesamiento de minerales, instalaciones de lixiviación, infraestructura eléctrica, sistemas de suministro de agua, caminos de acceso y alojamientos.</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1049,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1099,6 +1124,12 @@
       <color theme="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1222,21 +1253,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Notas" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="27">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="28">
     <dxf>
       <font>
         <strike val="0"/>
@@ -1282,7 +1299,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1432,6 +1449,26 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1518,12 +1555,12 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF212529"/>
         <name val="Times New Roman"/>
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1605,6 +1642,20 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <color rgb="FF212529"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
         <family val="1"/>
@@ -1670,38 +1721,40 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Lucas Ordoñez" id="{F2242E26-5684-4344-B202-B574D4AF1870}" userId="aece5baeefa9fdd6" providerId="Windows Live"/>
   <person displayName="Lucas Sebastian Ordoñez" id="{CC6B0CDD-571C-5947-AB3B-0FE73E1F689E}" userId="S::01OR42856583@campus.economicas.uba.ar::7e5516ec-a921-4253-95aa-4b0e13b66244" providerId="AD"/>
   <person displayName="Lucas Sebastian Ordoñez" id="{2E8DF262-CB25-3049-80AF-0C6513AADFB8}" userId="S::01or42856583@campus.economicas.uba.ar::7e5516ec-a921-4253-95aa-4b0e13b66244" providerId="AD"/>
 </personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProyectosIntegrados" displayName="ProyectosIntegrados" ref="A1:X40" headerRowDxfId="26" dataDxfId="0" totalsRowDxfId="25">
-  <tableColumns count="24">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="VPU" dataDxfId="24"/>
-    <tableColumn id="22" xr3:uid="{48F4E9CA-8EE4-9B46-B775-30029B62248E}" name="Descripción_del_proyecto" dataDxfId="23"/>
-    <tableColumn id="19" xr3:uid="{59A3C3BF-E3A1-3748-85BC-5ADA196D8039}" name="Proyectos de exportación estratégica de largo plazo (PEELP)" dataDxfId="22"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="id_proyecto" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="empresa" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="titular_proyecto" dataDxfId="19"/>
-    <tableColumn id="17" xr3:uid="{E1C7B229-46A1-4B4F-9ADD-A9E811939D67}" name="CUIT" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="sector" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="subsector" dataDxfId="16"/>
-    <tableColumn id="18" xr3:uid="{3AFF64F9-973D-4A41-865B-D4166A5841A1}" name="actividad_subsector_resolución_MECON" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="provincia" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="localidad_region" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Monto (mill. USD)" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Activos Computables (mill. USD)" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Estado administrativo" dataDxfId="10"/>
-    <tableColumn id="24" xr3:uid="{00D6C894-3563-A741-A5B5-7FF8DB602F8A}" name="Empleos (directos e indirectos)" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="fecha_presentacion" dataDxfId="8"/>
-    <tableColumn id="21" xr3:uid="{D27A2121-7D63-544C-B031-C3DB1A1B8B6A}" name="fecha_adhesion_rigi" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="fecha_publicacion_bo" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="norma_aprobacion" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{B0966B39-0FA3-9146-96DB-BD345771FAC8}" name="Clasificacion_preexistencia_boletin_oficial" dataDxfId="4"/>
-    <tableColumn id="23" xr3:uid="{36F41A70-CDCD-0440-8E79-C4973DF4F4B3}" name="Justificacion_preexistencia_boletin_oficial" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{BC53B1FB-4807-D244-BE0E-F220BF050122}" name="link_norma" dataDxfId="2"/>
-    <tableColumn id="20" xr3:uid="{6C16FCDF-822E-B843-A888-4F4B69680144}" name="Fuentes" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3BC5949B-99C1-C640-8DA2-C585B697BBE1}" name="ProyectosIntegrados2" displayName="ProyectosIntegrados2" ref="A1:Y40" headerRowDxfId="27" dataDxfId="26" totalsRowDxfId="25">
+  <tableColumns count="25">
+    <tableColumn id="2" xr3:uid="{1FB8F74D-9682-B440-94D1-B6000493E00B}" name="VPU" dataDxfId="24"/>
+    <tableColumn id="22" xr3:uid="{5F9EE6EB-2E4C-E743-B117-A1464438FFC7}" name="Descripción_del_proyecto" dataDxfId="23"/>
+    <tableColumn id="19" xr3:uid="{CFDF2429-F95D-3943-82F8-451A000B9F82}" name="Proyectos de exportación estratégica de largo plazo (PEELP)" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{AD64BC74-95BA-9A4E-AC4B-3DE73836DF90}" name="id_proyecto" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{51791E87-341F-3E41-878A-791662F5DBC9}" name="empresa" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{EADE9DE9-6117-8647-8338-D28DBAA6E72A}" name="titular_proyecto" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{904FDB28-DA1F-0547-8978-EB97CA045828}" name="CUIT" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{2D7A2D94-3733-994A-982A-DEDF8271CB6C}" name="sector" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{492831FB-44CE-CB47-B672-3D25B8F10010}" name="subsector" dataDxfId="16"/>
+    <tableColumn id="18" xr3:uid="{2D9EE4A5-6D6B-0047-8C2F-450DC201B187}" name="actividad_subsector_resolución_MECON" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{5BE522C7-9388-8F44-946E-83E19B93BC7A}" name="provincia" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{4E3CB780-5074-FA4F-B98A-31E67E04A07F}" name="localidad_region" dataDxfId="13"/>
+    <tableColumn id="25" xr3:uid="{00D4308B-7D36-6741-B428-F839A6601293}" name="Monto (mill. USD)" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{00FC2C60-51B2-5A4E-8D40-F20AEB84CDFF}" name="Monto (mill. USD) - aprobados resolución" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{A666CB24-8E9B-1A47-B550-E880F1AA03B2}" name="Activos Computables (mill. USD)" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{933A8A58-B5F6-224E-82E5-38224B7039BF}" name="Estado administrativo" dataDxfId="9"/>
+    <tableColumn id="24" xr3:uid="{D74832FC-F160-7B4E-B861-458D7BE39728}" name="Empleos (directos e indirectos)" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{1E31A58A-1B53-7345-B5A3-DDC3DE7DC28F}" name="fecha_presentacion" dataDxfId="7"/>
+    <tableColumn id="21" xr3:uid="{2EC6C086-DEA7-7148-A622-467B3FC9C8E5}" name="fecha_adhesion_rigi" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{1FBCC2F8-A44E-EE4B-B919-FD06CDA903B1}" name="fecha_publicacion_bo" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{AB9E3FD5-D9E1-FB4C-805E-4DC1E2E4F884}" name="norma_aprobacion" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{32A3F66C-F383-6A4F-BC9B-CE60E9775140}" name="Clasificacion_preexistencia_boletin_oficial" dataDxfId="3"/>
+    <tableColumn id="23" xr3:uid="{8FFE7748-3D7D-F44F-9EE0-37998D10E3B7}" name="Justificacion_preexistencia_boletin_oficial" dataDxfId="2"/>
+    <tableColumn id="16" xr3:uid="{B5F0282B-C127-7C40-86CC-663CD39DAAF5}" name="link_norma" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{4245686F-374C-B840-9963-4B9AF6D5BD62}" name="Fuentes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1883,15 +1936,22 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="E1" dT="2026-06-15T21:16:51.15" personId="{CC6B0CDD-571C-5947-AB3B-0FE73E1F689E}" id="{DBA8E842-1B69-4E44-955F-86A6656A5A38}">
+  <threadedComment ref="E1" dT="2026-06-15T21:16:51.15" personId="{CC6B0CDD-571C-5947-AB3B-0FE73E1F689E}" id="{CC7FC192-DD2F-524F-965B-B519233399BD}">
     <text xml:space="preserve">La fuente de datos de esta variable es el tracker de GLOBARIS
 </text>
   </threadedComment>
-  <threadedComment ref="P1" dT="2026-06-15T21:15:54.67" personId="{CC6B0CDD-571C-5947-AB3B-0FE73E1F689E}" id="{2603CD78-4DA2-7245-9496-2BEE29538FD4}">
+  <threadedComment ref="M1" dT="2026-07-30T19:12:39.35" personId="{F2242E26-5684-4344-B202-B574D4AF1870}" id="{EA61046C-C94E-C449-8761-ABD505A37332}">
+    <text xml:space="preserve">En los casos en que el monto total de inversión informado en el sitio web oficial del RIGI difiere del consignado en la resolución correspondiente a cada proyecto aprobado, se utiliza el monto publicado en el sitio web oficial del régimen.
+</text>
+  </threadedComment>
+  <threadedComment ref="N1" dT="2026-07-30T19:10:18.02" personId="{F2242E26-5684-4344-B202-B574D4AF1870}" id="{9E845984-16BC-D640-8568-DCBC39BD282B}">
+    <text>Se completo los datos de inversión total de los proyectos aprobados con los montos reportados en la resolución respectiva de cada proyecto. En algunos casos los montos reportados difieren en comparación a los reportados en el sitio web oficial del RIGI del gobierno</text>
+  </threadedComment>
+  <threadedComment ref="Q1" dT="2026-06-15T21:15:54.67" personId="{CC6B0CDD-571C-5947-AB3B-0FE73E1F689E}" id="{D756854B-3370-2C47-8E59-D458EBCA5109}">
     <text xml:space="preserve">La fuente de datos de esta variable es el monitor del RIGI del MECON
 </text>
   </threadedComment>
-  <threadedComment ref="M3" dT="2026-06-09T13:10:11.61" personId="{2E8DF262-CB25-3049-80AF-0C6513AADFB8}" id="{D89771A4-99A8-0740-A054-82109EE9B8C1}">
+  <threadedComment ref="N3" dT="2026-06-09T13:10:11.61" personId="{2E8DF262-CB25-3049-80AF-0C6513AADFB8}" id="{909B81E5-AB38-BB4F-A77E-C63D2711848A}">
     <text xml:space="preserve">Que el solicitante declaró que el proyecto implicará una inversión total de entre dólares estadounidenses dos mil novecientos millones (USD 2.900.000.000) y dólares estadounidenses tres mil doscientos millones (USD 3.200.000.000). Se computa el promedio
 </text>
   </threadedComment>
@@ -1900,13 +1960,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X49"/>
+  <dimension ref="A1:Y49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="94.33203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="16384" width="94.33203125" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>196</v>
       </c>
@@ -1914,7 +1974,7 @@
         <v>183</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
@@ -1947,45 +2007,48 @@
         <v>146</v>
       </c>
       <c r="N1" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="X1" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="Y1" s="7" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="30" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.15">
       <c r="A2" s="7" t="s">
         <v>40</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>169</v>
@@ -2018,48 +2081,51 @@
         <v>12</v>
       </c>
       <c r="M2" s="9">
+        <v>15156</v>
+      </c>
+      <c r="N2" s="9">
         <v>6878</v>
       </c>
-      <c r="N2" s="9">
+      <c r="O2" s="9">
         <v>2825</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="P2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="7">
+      <c r="Q2" s="7">
         <v>836</v>
       </c>
-      <c r="Q2" s="10">
+      <c r="R2" s="10">
         <v>45617</v>
       </c>
-      <c r="R2" s="10">
+      <c r="S2" s="10">
         <v>45775</v>
       </c>
-      <c r="S2" s="10">
+      <c r="T2" s="10">
         <v>45776</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="U2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="U2" s="7" t="s">
+      <c r="V2" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V2" s="7" t="s">
+      <c r="W2" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="W2" s="11" t="s">
+      <c r="X2" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="X2" s="7" t="s">
+      <c r="Y2" s="7" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
         <v>176</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>169</v>
@@ -2092,48 +2158,51 @@
         <v>12</v>
       </c>
       <c r="M3" s="9">
+        <v>2900</v>
+      </c>
+      <c r="N3" s="9">
         <v>3050</v>
       </c>
-      <c r="N3" s="9">
+      <c r="O3" s="9">
         <v>2486</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="P3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="7">
+      <c r="Q3" s="7">
         <v>3108</v>
       </c>
-      <c r="Q3" s="10">
+      <c r="R3" s="10">
         <v>45611</v>
       </c>
-      <c r="R3" s="10">
+      <c r="S3" s="10">
         <v>45722</v>
       </c>
-      <c r="S3" s="10">
+      <c r="T3" s="10">
         <v>45736</v>
       </c>
-      <c r="T3" s="7" t="s">
+      <c r="U3" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="U3" s="7" t="s">
+      <c r="V3" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V3" s="7" t="s">
+      <c r="W3" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="W3" s="12" t="s">
+      <c r="X3" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="X3" s="7" t="s">
+      <c r="Y3" s="7" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A4" s="7" t="s">
         <v>181</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>169</v>
@@ -2169,45 +2238,48 @@
         <v>2672.1709999999998</v>
       </c>
       <c r="N4" s="9">
+        <v>2672.1709999999998</v>
+      </c>
+      <c r="O4" s="9">
         <v>2354</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="P4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P4" s="7">
+      <c r="Q4" s="7">
         <v>7391</v>
       </c>
-      <c r="Q4" s="10">
+      <c r="R4" s="10">
         <v>45849</v>
       </c>
-      <c r="R4" s="10">
+      <c r="S4" s="10">
         <v>45925</v>
       </c>
-      <c r="S4" s="10">
+      <c r="T4" s="10">
         <v>45943</v>
       </c>
-      <c r="T4" s="7" t="s">
+      <c r="U4" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="U4" s="7" t="s">
+      <c r="V4" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="V4" s="7" t="s">
+      <c r="W4" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="W4" s="12" t="s">
+      <c r="X4" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="X4" s="7" t="s">
+      <c r="Y4" s="7" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="60" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:25" ht="60" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
         <v>185</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>169</v>
@@ -2243,40 +2315,43 @@
         <v>2744</v>
       </c>
       <c r="N5" s="9">
+        <v>2744</v>
+      </c>
+      <c r="O5" s="9">
         <v>2299</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="P5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P5" s="7">
+      <c r="Q5" s="7">
         <v>1985</v>
       </c>
-      <c r="Q5" s="10">
+      <c r="R5" s="10">
         <v>45713</v>
       </c>
-      <c r="R5" s="10">
+      <c r="S5" s="10">
         <v>45796</v>
       </c>
-      <c r="S5" s="10">
+      <c r="T5" s="10">
         <v>45807</v>
       </c>
-      <c r="T5" s="7" t="s">
+      <c r="U5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="U5" s="7" t="s">
+      <c r="V5" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="W5" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="W5" s="12" t="s">
+      <c r="X5" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="X5" s="7" t="s">
+      <c r="Y5" s="7" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
         <v>49</v>
       </c>
@@ -2314,48 +2389,51 @@
         <v>26</v>
       </c>
       <c r="M6" s="9">
-        <v>613.42999999999995</v>
+        <v>891</v>
       </c>
       <c r="N6" s="9">
         <v>613.42999999999995</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="O6" s="9">
+        <v>613.42999999999995</v>
+      </c>
+      <c r="P6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P6" s="7">
+      <c r="Q6" s="7">
         <v>6300</v>
       </c>
-      <c r="Q6" s="10">
+      <c r="R6" s="10">
         <v>45967</v>
       </c>
-      <c r="R6" s="10">
+      <c r="S6" s="10">
         <v>46155</v>
       </c>
-      <c r="S6" s="10">
+      <c r="T6" s="10">
         <v>46168</v>
       </c>
-      <c r="T6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="U6" s="7" t="s">
+      <c r="V6" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V6" s="7" t="s">
+      <c r="W6" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="W6" s="12" t="s">
+      <c r="X6" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="X6" s="7" t="s">
+      <c r="Y6" s="7" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
         <v>191</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>182</v>
@@ -2388,48 +2466,51 @@
         <v>26</v>
       </c>
       <c r="M7" s="9">
-        <v>519.64700000000005</v>
+        <v>665</v>
       </c>
       <c r="N7" s="9">
         <v>519.64700000000005</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="9">
+        <v>519.64700000000005</v>
+      </c>
+      <c r="P7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P7" s="7">
+      <c r="Q7" s="7">
         <v>4500</v>
       </c>
-      <c r="Q7" s="10">
+      <c r="R7" s="10">
         <v>45814</v>
       </c>
-      <c r="R7" s="10">
+      <c r="S7" s="10">
         <v>45988</v>
       </c>
-      <c r="S7" s="10">
+      <c r="T7" s="10">
         <v>46035</v>
       </c>
-      <c r="T7" s="7" t="s">
+      <c r="U7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="U7" s="7" t="s">
+      <c r="V7" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V7" s="13" t="s">
+      <c r="W7" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="W7" s="12" t="s">
+      <c r="X7" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="X7" s="7" t="s">
+      <c r="Y7" s="7" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
         <v>192</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>182</v>
@@ -2465,45 +2546,48 @@
         <v>550</v>
       </c>
       <c r="N8" s="9">
+        <v>550</v>
+      </c>
+      <c r="O8" s="9">
         <v>513.37199999999996</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="P8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P8" s="7">
+      <c r="Q8" s="7">
         <v>7535</v>
       </c>
-      <c r="Q8" s="10">
+      <c r="R8" s="10">
         <v>45957</v>
       </c>
-      <c r="R8" s="10">
+      <c r="S8" s="10">
         <v>46142</v>
       </c>
-      <c r="S8" s="10">
+      <c r="T8" s="10">
         <v>46154</v>
       </c>
-      <c r="T8" s="7" t="s">
+      <c r="U8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="U8" s="7" t="s">
+      <c r="V8" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="V8" s="7" t="s">
+      <c r="W8" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="W8" s="12" t="s">
+      <c r="X8" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="X8" s="7" t="s">
+      <c r="Y8" s="7" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>182</v>
@@ -2536,43 +2620,46 @@
         <v>21</v>
       </c>
       <c r="M9" s="9">
-        <v>481.7</v>
+        <v>764</v>
       </c>
       <c r="N9" s="9">
         <v>481.7</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="9">
+        <v>481.7</v>
+      </c>
+      <c r="P9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P9" s="7">
+      <c r="Q9" s="7">
         <v>2013</v>
       </c>
-      <c r="Q9" s="10">
+      <c r="R9" s="10">
         <v>45981</v>
       </c>
-      <c r="R9" s="10">
+      <c r="S9" s="10">
         <v>46080</v>
       </c>
-      <c r="S9" s="10">
+      <c r="T9" s="10">
         <v>46149</v>
       </c>
-      <c r="T9" s="7" t="s">
+      <c r="U9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="U9" s="7" t="s">
+      <c r="V9" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V9" s="7" t="s">
+      <c r="W9" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="W9" s="15" t="s">
+      <c r="X9" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="X9" s="7" t="s">
+      <c r="Y9" s="7" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="75" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:25" ht="75" x14ac:dyDescent="0.15">
       <c r="A10" s="14" t="s">
         <v>203</v>
       </c>
@@ -2610,48 +2697,51 @@
         <v>26</v>
       </c>
       <c r="M10" s="9">
-        <v>380.11599999999999</v>
+        <v>436</v>
       </c>
       <c r="N10" s="9">
         <v>380.11599999999999</v>
       </c>
-      <c r="O10" s="7" t="s">
+      <c r="O10" s="9">
+        <v>380.11599999999999</v>
+      </c>
+      <c r="P10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P10" s="7">
+      <c r="Q10" s="7">
         <v>1048</v>
       </c>
-      <c r="Q10" s="10">
+      <c r="R10" s="10">
         <v>45873</v>
       </c>
-      <c r="R10" s="10">
+      <c r="S10" s="10">
         <v>46050</v>
       </c>
-      <c r="S10" s="10">
+      <c r="T10" s="10">
         <v>46111</v>
       </c>
-      <c r="T10" s="7" t="s">
+      <c r="U10" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="U10" s="14" t="s">
+      <c r="V10" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="V10" s="7" t="s">
+      <c r="W10" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="W10" s="15" t="s">
+      <c r="X10" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="X10" s="7" t="s">
+      <c r="Y10" s="7" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="75" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:25" ht="75" x14ac:dyDescent="0.15">
       <c r="A11" s="7" t="s">
         <v>44</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>182</v>
@@ -2689,43 +2779,46 @@
       <c r="N11" s="9">
         <v>286.27800000000002</v>
       </c>
-      <c r="O11" s="7" t="s">
+      <c r="O11" s="9">
+        <v>286.27800000000002</v>
+      </c>
+      <c r="P11" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P11" s="7">
+      <c r="Q11" s="7">
         <v>3800</v>
       </c>
-      <c r="Q11" s="10">
+      <c r="R11" s="10">
         <v>45638</v>
       </c>
-      <c r="R11" s="10">
+      <c r="S11" s="10">
         <v>45807</v>
       </c>
-      <c r="S11" s="10">
+      <c r="T11" s="10">
         <v>45859</v>
       </c>
-      <c r="T11" s="7" t="s">
+      <c r="U11" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="U11" s="7" t="s">
+      <c r="V11" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V11" s="7" t="s">
+      <c r="W11" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="W11" s="11" t="s">
+      <c r="X11" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="X11" s="7" t="s">
+      <c r="Y11" s="7" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="60" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:25" ht="60" x14ac:dyDescent="0.15">
       <c r="A12" s="7" t="s">
         <v>210</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>182</v>
@@ -2763,43 +2856,46 @@
       <c r="N12" s="9">
         <v>276.89999999999998</v>
       </c>
-      <c r="O12" s="7" t="s">
+      <c r="O12" s="9">
+        <v>276.89999999999998</v>
+      </c>
+      <c r="P12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P12" s="7">
+      <c r="Q12" s="7">
         <v>9700</v>
       </c>
-      <c r="Q12" s="10">
+      <c r="R12" s="10">
         <v>45757</v>
       </c>
-      <c r="R12" s="10">
+      <c r="S12" s="10">
         <v>45953</v>
       </c>
-      <c r="S12" s="10">
+      <c r="T12" s="10">
         <v>45980</v>
       </c>
-      <c r="T12" s="7" t="s">
+      <c r="U12" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="U12" s="7" t="s">
+      <c r="V12" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V12" s="7" t="s">
+      <c r="W12" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="W12" s="12" t="s">
+      <c r="X12" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="X12" s="7" t="s">
+      <c r="Y12" s="7" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="120" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:25" ht="120" x14ac:dyDescent="0.15">
       <c r="A13" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>182</v>
@@ -2835,45 +2931,48 @@
         <v>275.58999999999997</v>
       </c>
       <c r="N13" s="9">
+        <v>275.58999999999997</v>
+      </c>
+      <c r="O13" s="9">
         <v>255.11199999999999</v>
       </c>
-      <c r="O13" s="7" t="s">
+      <c r="P13" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P13" s="7">
+      <c r="Q13" s="7">
         <v>165</v>
       </c>
-      <c r="Q13" s="10">
+      <c r="R13" s="10">
         <v>45656</v>
       </c>
-      <c r="R13" s="10">
+      <c r="S13" s="10">
         <v>45863</v>
       </c>
-      <c r="S13" s="10">
+      <c r="T13" s="10">
         <v>45895</v>
       </c>
-      <c r="T13" s="7" t="s">
+      <c r="U13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="U13" s="7" t="s">
+      <c r="V13" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V13" s="7" t="s">
+      <c r="W13" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="W13" s="12" t="s">
+      <c r="X13" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="X13" s="7" t="s">
+      <c r="Y13" s="7" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="120" x14ac:dyDescent="0.15">
-      <c r="A14" s="7" t="s">
-        <v>191</v>
+    <row r="14" spans="1:25" ht="120" x14ac:dyDescent="0.15">
+      <c r="A14" s="17" t="s">
+        <v>306</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>182</v>
@@ -2906,48 +3005,51 @@
         <v>21</v>
       </c>
       <c r="M14" s="9">
-        <v>251.321</v>
+        <v>531</v>
       </c>
       <c r="N14" s="9">
         <v>251.321</v>
       </c>
-      <c r="O14" s="7" t="s">
+      <c r="O14" s="9">
+        <v>251.321</v>
+      </c>
+      <c r="P14" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P14" s="7">
+      <c r="Q14" s="7">
         <v>1273</v>
       </c>
-      <c r="Q14" s="10">
+      <c r="R14" s="10">
         <v>45898</v>
       </c>
-      <c r="R14" s="10">
+      <c r="S14" s="10">
         <v>46106</v>
       </c>
-      <c r="S14" s="10">
+      <c r="T14" s="10">
         <v>46112</v>
       </c>
-      <c r="T14" s="7" t="s">
+      <c r="U14" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="U14" s="7" t="s">
+      <c r="V14" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="V14" s="7" t="s">
+      <c r="W14" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="W14" s="12" t="s">
+      <c r="X14" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="X14" s="7" t="s">
+      <c r="Y14" s="7" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A15" s="7" t="s">
         <v>71</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>182</v>
@@ -2980,48 +3082,51 @@
         <v>21</v>
       </c>
       <c r="M15" s="9">
-        <v>217.09</v>
+        <v>292</v>
       </c>
       <c r="N15" s="9">
         <v>217.09</v>
       </c>
-      <c r="O15" s="7" t="s">
+      <c r="O15" s="9">
+        <v>217.09</v>
+      </c>
+      <c r="P15" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P15" s="7">
+      <c r="Q15" s="7">
         <v>670</v>
       </c>
-      <c r="Q15" s="10">
+      <c r="R15" s="10">
         <v>45594</v>
       </c>
-      <c r="R15" s="10">
+      <c r="S15" s="10">
         <v>45855</v>
       </c>
-      <c r="S15" s="10">
+      <c r="T15" s="10">
         <v>45896</v>
       </c>
-      <c r="T15" s="7" t="s">
+      <c r="U15" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="U15" s="7" t="s">
+      <c r="V15" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V15" s="7" t="s">
+      <c r="W15" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="W15" s="12" t="s">
+      <c r="X15" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="X15" s="7" t="s">
+      <c r="Y15" s="7" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A16" s="7" t="s">
         <v>35</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>182</v>
@@ -3052,43 +3157,46 @@
         <v>26</v>
       </c>
       <c r="M16" s="9">
-        <v>211.6</v>
+        <v>211</v>
       </c>
       <c r="N16" s="9">
-        <v>211.6</v>
-      </c>
-      <c r="O16" s="7" t="s">
+        <v>211.60007200000001</v>
+      </c>
+      <c r="O16" s="9">
+        <v>211.60007200000001</v>
+      </c>
+      <c r="P16" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P16" s="7">
+      <c r="Q16" s="7">
         <v>384</v>
       </c>
-      <c r="Q16" s="10">
+      <c r="R16" s="10">
         <v>45590</v>
       </c>
-      <c r="R16" s="10">
+      <c r="S16" s="10">
         <v>45642</v>
       </c>
-      <c r="S16" s="10">
+      <c r="T16" s="10">
         <v>45664</v>
       </c>
-      <c r="T16" s="7" t="s">
+      <c r="U16" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="U16" s="7" t="s">
+      <c r="V16" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="V16" s="13" t="s">
+      <c r="W16" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="W16" s="12" t="s">
+      <c r="X16" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="X16" s="7" t="s">
+      <c r="Y16" s="7" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A17" s="7" t="s">
         <v>78</v>
       </c>
@@ -3120,25 +3228,28 @@
       <c r="M17" s="9">
         <v>726</v>
       </c>
-      <c r="N17" s="9"/>
-      <c r="O17" s="7" t="s">
+      <c r="N17" s="9">
+        <v>726</v>
+      </c>
+      <c r="O17" s="9"/>
+      <c r="P17" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="10">
+      <c r="Q17" s="7"/>
+      <c r="R17" s="10">
         <v>45671</v>
       </c>
-      <c r="R17" s="10"/>
       <c r="S17" s="10"/>
-      <c r="T17" s="7"/>
+      <c r="T17" s="10"/>
       <c r="U17" s="7"/>
       <c r="V17" s="7"/>
-      <c r="W17" s="12"/>
-      <c r="X17" s="7" t="s">
+      <c r="W17" s="7"/>
+      <c r="X17" s="12"/>
+      <c r="Y17" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A18" s="7" t="s">
         <v>81</v>
       </c>
@@ -3170,25 +3281,28 @@
       <c r="M18" s="9">
         <v>232</v>
       </c>
-      <c r="N18" s="9"/>
-      <c r="O18" s="7" t="s">
+      <c r="N18" s="9">
+        <v>232</v>
+      </c>
+      <c r="O18" s="9"/>
+      <c r="P18" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="10">
+      <c r="Q18" s="7"/>
+      <c r="R18" s="10">
         <v>45874</v>
       </c>
-      <c r="R18" s="10"/>
       <c r="S18" s="10"/>
-      <c r="T18" s="7"/>
+      <c r="T18" s="10"/>
       <c r="U18" s="7"/>
       <c r="V18" s="7"/>
-      <c r="W18" s="15"/>
-      <c r="X18" s="7" t="s">
+      <c r="W18" s="7"/>
+      <c r="X18" s="15"/>
+      <c r="Y18" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="19" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A19" s="14" t="s">
         <v>86</v>
       </c>
@@ -3220,25 +3334,28 @@
       <c r="M19" s="9">
         <v>12000</v>
       </c>
-      <c r="N19" s="9"/>
-      <c r="O19" s="7" t="s">
+      <c r="N19" s="9">
+        <v>12000</v>
+      </c>
+      <c r="O19" s="9"/>
+      <c r="P19" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="10">
+      <c r="Q19" s="7"/>
+      <c r="R19" s="10">
         <v>45771</v>
       </c>
-      <c r="R19" s="10"/>
       <c r="S19" s="10"/>
-      <c r="T19" s="7"/>
+      <c r="T19" s="10"/>
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
-      <c r="W19" s="15"/>
-      <c r="X19" s="7" t="s">
+      <c r="W19" s="7"/>
+      <c r="X19" s="15"/>
+      <c r="Y19" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="45" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A20" s="7" t="s">
         <v>219</v>
       </c>
@@ -3276,43 +3393,46 @@
         <v>21</v>
       </c>
       <c r="M20" s="9">
-        <v>1166.6777259999999</v>
+        <v>1241</v>
       </c>
       <c r="N20" s="9">
         <v>1166.6777259999999</v>
       </c>
-      <c r="O20" s="7" t="s">
+      <c r="O20" s="9">
+        <v>1166.6777259999999</v>
+      </c>
+      <c r="P20" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P20" s="7">
+      <c r="Q20" s="7">
         <v>1787</v>
       </c>
-      <c r="Q20" s="10">
+      <c r="R20" s="10">
         <v>45795</v>
       </c>
-      <c r="R20" s="10">
+      <c r="S20" s="10">
         <v>46151</v>
       </c>
-      <c r="S20" s="10">
+      <c r="T20" s="10">
         <v>46177</v>
       </c>
-      <c r="T20" s="7" t="s">
+      <c r="U20" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="U20" s="7" t="s">
+      <c r="V20" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="V20" s="7" t="s">
+      <c r="W20" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="W20" s="15" t="s">
+      <c r="X20" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="X20" s="7" t="s">
+      <c r="Y20" s="7" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A21" s="14" t="s">
         <v>92</v>
       </c>
@@ -3344,25 +3464,28 @@
       <c r="M21" s="9">
         <v>380</v>
       </c>
-      <c r="N21" s="9"/>
-      <c r="O21" s="7" t="s">
+      <c r="N21" s="9">
+        <v>380</v>
+      </c>
+      <c r="O21" s="9"/>
+      <c r="P21" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="10">
+      <c r="Q21" s="7"/>
+      <c r="R21" s="10">
         <v>45859</v>
       </c>
-      <c r="R21" s="10"/>
       <c r="S21" s="10"/>
-      <c r="T21" s="7"/>
+      <c r="T21" s="10"/>
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
-      <c r="W21" s="15"/>
-      <c r="X21" s="7" t="s">
+      <c r="W21" s="7"/>
+      <c r="X21" s="15"/>
+      <c r="Y21" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A22" s="7" t="s">
         <v>95</v>
       </c>
@@ -3394,25 +3517,28 @@
       <c r="M22" s="9">
         <v>9500</v>
       </c>
-      <c r="N22" s="9"/>
-      <c r="O22" s="7" t="s">
+      <c r="N22" s="9">
+        <v>9500</v>
+      </c>
+      <c r="O22" s="9"/>
+      <c r="P22" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="10">
+      <c r="Q22" s="7"/>
+      <c r="R22" s="10">
         <v>45887</v>
       </c>
-      <c r="R22" s="10"/>
       <c r="S22" s="10"/>
-      <c r="T22" s="7"/>
+      <c r="T22" s="10"/>
       <c r="U22" s="7"/>
       <c r="V22" s="7"/>
-      <c r="W22" s="15"/>
-      <c r="X22" s="7" t="s">
+      <c r="W22" s="7"/>
+      <c r="X22" s="15"/>
+      <c r="Y22" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A23" s="13" t="s">
         <v>98</v>
       </c>
@@ -3444,25 +3570,28 @@
       <c r="M23" s="9">
         <v>13800</v>
       </c>
-      <c r="N23" s="9"/>
-      <c r="O23" s="7" t="s">
+      <c r="N23" s="9">
+        <v>13800</v>
+      </c>
+      <c r="O23" s="9"/>
+      <c r="P23" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="10">
+      <c r="Q23" s="7"/>
+      <c r="R23" s="10">
         <v>46175</v>
       </c>
-      <c r="R23" s="10"/>
       <c r="S23" s="10"/>
-      <c r="T23" s="7"/>
+      <c r="T23" s="10"/>
       <c r="U23" s="7"/>
       <c r="V23" s="7"/>
-      <c r="W23" s="15"/>
-      <c r="X23" s="7" t="s">
+      <c r="W23" s="7"/>
+      <c r="X23" s="15"/>
+      <c r="Y23" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A24" s="7" t="s">
         <v>136</v>
       </c>
@@ -3494,30 +3623,33 @@
       <c r="M24" s="9">
         <v>2400</v>
       </c>
-      <c r="N24" s="9"/>
-      <c r="O24" s="7" t="s">
+      <c r="N24" s="9">
+        <v>2400</v>
+      </c>
+      <c r="O24" s="9"/>
+      <c r="P24" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="10">
+      <c r="Q24" s="7"/>
+      <c r="R24" s="10">
         <v>46136</v>
       </c>
-      <c r="R24" s="10"/>
       <c r="S24" s="10"/>
-      <c r="T24" s="7"/>
+      <c r="T24" s="10"/>
       <c r="U24" s="7"/>
       <c r="V24" s="7"/>
-      <c r="W24" s="15"/>
-      <c r="X24" s="7" t="s">
+      <c r="W24" s="7"/>
+      <c r="X24" s="15"/>
+      <c r="Y24" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="90" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:25" ht="90" x14ac:dyDescent="0.15">
       <c r="A25" s="7" t="s">
         <v>263</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>182</v>
@@ -3553,40 +3685,43 @@
         <v>1300</v>
       </c>
       <c r="N25" s="9">
+        <v>1300</v>
+      </c>
+      <c r="O25" s="9">
         <v>955</v>
       </c>
-      <c r="O25" s="7" t="s">
+      <c r="P25" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P25" s="7">
+      <c r="Q25" s="7">
         <v>2489</v>
       </c>
-      <c r="Q25" s="10">
+      <c r="R25" s="10">
         <v>45950</v>
       </c>
-      <c r="R25" s="10">
+      <c r="S25" s="10">
         <v>46174</v>
       </c>
-      <c r="S25" s="10">
+      <c r="T25" s="10">
         <v>46198</v>
       </c>
-      <c r="T25" s="7" t="s">
+      <c r="U25" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="U25" s="7" t="s">
+      <c r="V25" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="V25" s="7" t="s">
+      <c r="W25" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="W25" s="12" t="s">
+      <c r="X25" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="X25" s="7" t="s">
+      <c r="Y25" s="7" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A26" s="7" t="s">
         <v>140</v>
       </c>
@@ -3618,25 +3753,28 @@
       <c r="M26" s="9">
         <v>1151</v>
       </c>
-      <c r="N26" s="9"/>
-      <c r="O26" s="7" t="s">
+      <c r="N26" s="9">
+        <v>1151</v>
+      </c>
+      <c r="O26" s="9"/>
+      <c r="P26" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="10">
+      <c r="Q26" s="7"/>
+      <c r="R26" s="10">
         <v>46111</v>
       </c>
-      <c r="R26" s="10"/>
       <c r="S26" s="10"/>
-      <c r="T26" s="7"/>
+      <c r="T26" s="10"/>
       <c r="U26" s="7"/>
       <c r="V26" s="7"/>
       <c r="W26" s="7"/>
-      <c r="X26" s="7" t="s">
+      <c r="X26" s="7"/>
+      <c r="Y26" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="27" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A27" s="7" t="s">
         <v>149</v>
       </c>
@@ -3668,25 +3806,28 @@
       <c r="M27" s="9">
         <v>25000</v>
       </c>
-      <c r="N27" s="9"/>
-      <c r="O27" s="7" t="s">
+      <c r="N27" s="9">
+        <v>25000</v>
+      </c>
+      <c r="O27" s="9"/>
+      <c r="P27" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="10">
+      <c r="Q27" s="7"/>
+      <c r="R27" s="10">
         <v>46157</v>
       </c>
-      <c r="R27" s="10"/>
       <c r="S27" s="10"/>
-      <c r="T27" s="7"/>
+      <c r="T27" s="10"/>
       <c r="U27" s="7"/>
       <c r="V27" s="7"/>
       <c r="W27" s="7"/>
-      <c r="X27" s="7" t="s">
+      <c r="X27" s="7"/>
+      <c r="Y27" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="28" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A28" s="7" t="s">
         <v>126</v>
       </c>
@@ -3718,25 +3859,28 @@
       <c r="M28" s="9">
         <v>1000</v>
       </c>
-      <c r="N28" s="9"/>
-      <c r="O28" s="7" t="s">
+      <c r="N28" s="9">
+        <v>1000</v>
+      </c>
+      <c r="O28" s="9"/>
+      <c r="P28" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="10">
+      <c r="Q28" s="7"/>
+      <c r="R28" s="10">
         <v>46157</v>
       </c>
-      <c r="R28" s="10"/>
       <c r="S28" s="10"/>
-      <c r="T28" s="7"/>
+      <c r="T28" s="10"/>
       <c r="U28" s="7"/>
       <c r="V28" s="7"/>
       <c r="W28" s="7"/>
-      <c r="X28" s="7" t="s">
+      <c r="X28" s="7"/>
+      <c r="Y28" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="29" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A29" s="14" t="s">
         <v>128</v>
       </c>
@@ -3768,25 +3912,28 @@
       <c r="M29" s="9">
         <v>273</v>
       </c>
-      <c r="N29" s="9"/>
-      <c r="O29" s="7" t="s">
+      <c r="N29" s="9">
+        <v>273</v>
+      </c>
+      <c r="O29" s="9"/>
+      <c r="P29" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="P29" s="7"/>
-      <c r="Q29" s="10">
+      <c r="Q29" s="7"/>
+      <c r="R29" s="10">
         <v>45717</v>
       </c>
-      <c r="R29" s="10"/>
       <c r="S29" s="10"/>
-      <c r="T29" s="7"/>
+      <c r="T29" s="10"/>
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="7"/>
-      <c r="X29" s="7" t="s">
+      <c r="X29" s="7"/>
+      <c r="Y29" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A30" s="7" t="s">
         <v>132</v>
       </c>
@@ -3818,25 +3965,28 @@
       <c r="M30" s="9">
         <v>360</v>
       </c>
-      <c r="N30" s="9"/>
-      <c r="O30" s="7" t="s">
+      <c r="N30" s="9">
+        <v>360</v>
+      </c>
+      <c r="O30" s="9"/>
+      <c r="P30" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P30" s="7"/>
-      <c r="Q30" s="10">
+      <c r="Q30" s="7"/>
+      <c r="R30" s="10">
         <v>46099</v>
       </c>
-      <c r="R30" s="10"/>
       <c r="S30" s="10"/>
-      <c r="T30" s="7"/>
+      <c r="T30" s="10"/>
       <c r="U30" s="7"/>
       <c r="V30" s="7"/>
       <c r="W30" s="7"/>
-      <c r="X30" s="7" t="s">
+      <c r="X30" s="7"/>
+      <c r="Y30" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="31" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A31" s="7" t="s">
         <v>134</v>
       </c>
@@ -3868,25 +4018,28 @@
       <c r="M31" s="9">
         <v>4000</v>
       </c>
-      <c r="N31" s="9"/>
-      <c r="O31" s="7" t="s">
+      <c r="N31" s="9">
+        <v>4000</v>
+      </c>
+      <c r="O31" s="9"/>
+      <c r="P31" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="10">
+      <c r="Q31" s="7"/>
+      <c r="R31" s="10">
         <v>45887</v>
       </c>
-      <c r="R31" s="10"/>
       <c r="S31" s="10"/>
-      <c r="T31" s="7"/>
+      <c r="T31" s="10"/>
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
-      <c r="X31" s="7" t="s">
+      <c r="X31" s="7"/>
+      <c r="Y31" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="32" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A32" s="7" t="s">
         <v>100</v>
       </c>
@@ -3918,25 +4071,28 @@
       <c r="M32" s="9">
         <v>200</v>
       </c>
-      <c r="N32" s="9"/>
-      <c r="O32" s="7" t="s">
+      <c r="N32" s="9">
+        <v>200</v>
+      </c>
+      <c r="O32" s="9"/>
+      <c r="P32" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P32" s="7"/>
-      <c r="Q32" s="10" t="s">
+      <c r="Q32" s="7"/>
+      <c r="R32" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="R32" s="10"/>
       <c r="S32" s="10"/>
-      <c r="T32" s="7"/>
+      <c r="T32" s="10"/>
       <c r="U32" s="7"/>
       <c r="V32" s="7"/>
       <c r="W32" s="7"/>
-      <c r="X32" s="7" t="s">
+      <c r="X32" s="7"/>
+      <c r="Y32" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="33" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A33" s="7" t="s">
         <v>105</v>
       </c>
@@ -3968,25 +4124,28 @@
       <c r="M33" s="9">
         <v>206</v>
       </c>
-      <c r="N33" s="9"/>
-      <c r="O33" s="7" t="s">
+      <c r="N33" s="9">
+        <v>206</v>
+      </c>
+      <c r="O33" s="9"/>
+      <c r="P33" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="10">
+      <c r="Q33" s="7"/>
+      <c r="R33" s="10">
         <v>45805</v>
       </c>
-      <c r="R33" s="10"/>
       <c r="S33" s="10"/>
-      <c r="T33" s="7"/>
+      <c r="T33" s="10"/>
       <c r="U33" s="7"/>
       <c r="V33" s="7"/>
       <c r="W33" s="7"/>
-      <c r="X33" s="7" t="s">
+      <c r="X33" s="7"/>
+      <c r="Y33" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="34" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A34" s="7" t="s">
         <v>108</v>
       </c>
@@ -4018,25 +4177,28 @@
       <c r="M34" s="9">
         <v>6391</v>
       </c>
-      <c r="N34" s="9"/>
-      <c r="O34" s="7" t="s">
+      <c r="N34" s="9">
+        <v>6391</v>
+      </c>
+      <c r="O34" s="9"/>
+      <c r="P34" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P34" s="7"/>
-      <c r="Q34" s="10">
+      <c r="Q34" s="7"/>
+      <c r="R34" s="10">
         <v>46118</v>
       </c>
-      <c r="R34" s="10"/>
       <c r="S34" s="10"/>
-      <c r="T34" s="7"/>
+      <c r="T34" s="10"/>
       <c r="U34" s="7"/>
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
-      <c r="X34" s="7" t="s">
+      <c r="X34" s="7"/>
+      <c r="Y34" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="35" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A35" s="7" t="s">
         <v>111</v>
       </c>
@@ -4068,30 +4230,33 @@
       <c r="M35" s="9">
         <v>4245</v>
       </c>
-      <c r="N35" s="9"/>
-      <c r="O35" s="7" t="s">
+      <c r="N35" s="9">
+        <v>4245</v>
+      </c>
+      <c r="O35" s="9"/>
+      <c r="P35" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P35" s="7"/>
-      <c r="Q35" s="10">
+      <c r="Q35" s="7"/>
+      <c r="R35" s="10">
         <v>46081</v>
       </c>
-      <c r="R35" s="10"/>
       <c r="S35" s="10"/>
-      <c r="T35" s="7"/>
+      <c r="T35" s="10"/>
       <c r="U35" s="7"/>
       <c r="V35" s="7"/>
       <c r="W35" s="7"/>
-      <c r="X35" s="7" t="s">
+      <c r="X35" s="7"/>
+      <c r="Y35" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="90" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:25" ht="90" x14ac:dyDescent="0.15">
       <c r="A36" s="7" t="s">
         <v>270</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>169</v>
@@ -4106,7 +4271,7 @@
         <v>115</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H36" s="9" t="s">
         <v>165</v>
@@ -4115,7 +4280,7 @@
         <v>165</v>
       </c>
       <c r="J36" s="17" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>89</v>
@@ -4124,43 +4289,46 @@
         <v>12</v>
       </c>
       <c r="M36" s="9">
-        <v>4521</v>
+        <v>4522</v>
       </c>
       <c r="N36" s="9">
         <v>4521</v>
       </c>
-      <c r="O36" s="7" t="s">
+      <c r="O36" s="9">
+        <v>4521</v>
+      </c>
+      <c r="P36" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P36" s="7">
+      <c r="Q36" s="7">
         <v>1733</v>
       </c>
-      <c r="Q36" s="10">
+      <c r="R36" s="10">
         <v>46090</v>
       </c>
-      <c r="R36" s="10">
+      <c r="S36" s="10">
         <v>46198</v>
       </c>
-      <c r="S36" s="10">
+      <c r="T36" s="10">
         <v>46224</v>
       </c>
-      <c r="T36" s="7" t="s">
-        <v>273</v>
-      </c>
       <c r="U36" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="V36" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="V36" s="16" t="s">
-        <v>277</v>
-      </c>
-      <c r="W36" s="7" t="s">
+      <c r="W36" s="16" t="s">
+        <v>276</v>
+      </c>
+      <c r="X36" s="15" t="s">
         <v>272</v>
       </c>
-      <c r="X36" s="7" t="s">
+      <c r="Y36" s="7" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="37" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A37" s="7" t="s">
         <v>116</v>
       </c>
@@ -4192,25 +4360,28 @@
       <c r="M37" s="9">
         <v>845</v>
       </c>
-      <c r="N37" s="9"/>
-      <c r="O37" s="7" t="s">
+      <c r="N37" s="9">
+        <v>845</v>
+      </c>
+      <c r="O37" s="9"/>
+      <c r="P37" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="10">
+      <c r="Q37" s="7"/>
+      <c r="R37" s="10">
         <v>45595</v>
       </c>
-      <c r="R37" s="10"/>
       <c r="S37" s="10"/>
-      <c r="T37" s="7"/>
+      <c r="T37" s="10"/>
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
       <c r="W37" s="7"/>
-      <c r="X37" s="7" t="s">
+      <c r="X37" s="7"/>
+      <c r="Y37" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="38" spans="1:24" ht="15" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A38" s="7" t="s">
         <v>119</v>
       </c>
@@ -4242,30 +4413,33 @@
       <c r="M38" s="9">
         <v>818</v>
       </c>
-      <c r="N38" s="9"/>
-      <c r="O38" s="7" t="s">
+      <c r="N38" s="9">
+        <v>818</v>
+      </c>
+      <c r="O38" s="9"/>
+      <c r="P38" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="P38" s="7"/>
-      <c r="Q38" s="10">
+      <c r="Q38" s="7"/>
+      <c r="R38" s="10">
         <v>45758</v>
       </c>
-      <c r="R38" s="10"/>
       <c r="S38" s="10"/>
-      <c r="T38" s="7"/>
+      <c r="T38" s="10"/>
       <c r="U38" s="7"/>
       <c r="V38" s="7"/>
       <c r="W38" s="7"/>
-      <c r="X38" s="7" t="s">
+      <c r="X38" s="7"/>
+      <c r="Y38" s="7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="39" spans="1:24" ht="90" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:25" ht="90" x14ac:dyDescent="0.15">
       <c r="A39" s="17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C39" s="7"/>
       <c r="D39" s="8">
@@ -4278,7 +4452,7 @@
         <v>122</v>
       </c>
       <c r="G39" s="17" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H39" s="9" t="s">
         <v>19</v>
@@ -4299,45 +4473,48 @@
         <v>710</v>
       </c>
       <c r="N39" s="9">
+        <v>710</v>
+      </c>
+      <c r="O39" s="9">
         <v>594.13599999999997</v>
       </c>
-      <c r="O39" s="7" t="s">
+      <c r="P39" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P39" s="7">
+      <c r="Q39" s="7">
         <v>4406</v>
       </c>
-      <c r="Q39" s="10">
+      <c r="R39" s="10">
         <v>46063</v>
       </c>
-      <c r="R39" s="10">
+      <c r="S39" s="10">
         <v>46206</v>
       </c>
-      <c r="S39" s="10">
+      <c r="T39" s="10">
         <v>46232</v>
       </c>
-      <c r="T39" s="7" t="s">
-        <v>281</v>
-      </c>
       <c r="U39" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="V39" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="V39" s="16" t="s">
-        <v>284</v>
-      </c>
-      <c r="W39" s="7" t="s">
-        <v>280</v>
-      </c>
-      <c r="X39" s="7" t="s">
+      <c r="W39" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="X39" s="15" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="40" spans="1:24" ht="90" x14ac:dyDescent="0.15">
+      <c r="Y39" s="7" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25" ht="90" x14ac:dyDescent="0.15">
       <c r="A40" s="17" t="s">
         <v>123</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>169</v>
@@ -4352,13 +4529,13 @@
         <v>125</v>
       </c>
       <c r="G40" s="17" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H40" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J40" s="14" t="s">
         <v>179</v>
@@ -4373,40 +4550,43 @@
         <v>9737.0139999999992</v>
       </c>
       <c r="N40" s="9">
+        <v>9737.0139999999992</v>
+      </c>
+      <c r="O40" s="9">
         <v>9024.7322810000005</v>
       </c>
-      <c r="O40" s="7" t="s">
+      <c r="P40" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="P40" s="7">
-        <v>30000</v>
-      </c>
-      <c r="Q40" s="10">
+      <c r="Q40" s="7">
+        <v>31700</v>
+      </c>
+      <c r="R40" s="10">
         <v>46002</v>
       </c>
-      <c r="R40" s="10">
+      <c r="S40" s="10">
         <v>46176</v>
       </c>
-      <c r="S40" s="10">
+      <c r="T40" s="10">
         <v>46233</v>
       </c>
-      <c r="T40" s="7" t="s">
+      <c r="U40" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="V40" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="W40" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="X40" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="Y40" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="U40" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="V40" s="16" t="s">
-        <v>306</v>
-      </c>
-      <c r="W40" s="15" t="s">
-        <v>304</v>
-      </c>
-      <c r="X40" s="7" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.15">
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A41" s="7"/>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
@@ -4432,7 +4612,7 @@
       <c r="W41" s="7"/>
       <c r="X41" s="7"/>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A42" s="7"/>
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
@@ -4458,7 +4638,7 @@
       <c r="W42" s="7"/>
       <c r="X42" s="7"/>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
@@ -4484,7 +4664,7 @@
       <c r="W43" s="7"/>
       <c r="X43" s="7"/>
     </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -4510,7 +4690,7 @@
       <c r="W44" s="7"/>
       <c r="X44" s="7"/>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
@@ -4536,7 +4716,7 @@
       <c r="W45" s="7"/>
       <c r="X45" s="7"/>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
@@ -4562,7 +4742,7 @@
       <c r="W46" s="7"/>
       <c r="X46" s="7"/>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
@@ -4588,7 +4768,7 @@
       <c r="W47" s="7"/>
       <c r="X47" s="7"/>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
@@ -4643,28 +4823,30 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="W16" r:id="rId1" xr:uid="{980A8705-7984-584F-AA67-D26C392ABC82}"/>
-    <hyperlink ref="W2" r:id="rId2" xr:uid="{9D626AFB-AED7-6E45-B753-789A1F6791C1}"/>
-    <hyperlink ref="W3" r:id="rId3" xr:uid="{C1F9917A-BBEE-3848-A846-5585A2FCCC16}"/>
-    <hyperlink ref="W4" r:id="rId4" xr:uid="{E61BB65B-5618-D842-B6B5-1D004A053D60}"/>
-    <hyperlink ref="W5" r:id="rId5" xr:uid="{030CB02F-3E38-AE45-AC1C-EE5651975CBA}"/>
-    <hyperlink ref="W6" r:id="rId6" xr:uid="{232A6A28-624D-CE40-BFCA-AD0E1FB7DF56}"/>
-    <hyperlink ref="W7" r:id="rId7" xr:uid="{C26CF64B-E057-8241-B386-6B0B94FD84CC}"/>
-    <hyperlink ref="W8" r:id="rId8" xr:uid="{FF6237C1-652C-1A4A-B04E-3FB26C32DBD5}"/>
-    <hyperlink ref="W9" r:id="rId9" xr:uid="{FE5C09BA-9D83-1C4D-A289-7D742AB36DC4}"/>
-    <hyperlink ref="W10" r:id="rId10" xr:uid="{28CFDF16-2940-5642-9869-C1E5F4C077CE}"/>
-    <hyperlink ref="W11" r:id="rId11" xr:uid="{C215718F-64A5-EA4F-8EA7-85C30B114214}"/>
-    <hyperlink ref="W12" r:id="rId12" xr:uid="{BE9CC28B-94CE-B24E-A74E-3D2ADB3217C6}"/>
-    <hyperlink ref="W13" r:id="rId13" xr:uid="{66457491-26B9-9F44-8331-CABFE31C9F72}"/>
-    <hyperlink ref="W14" r:id="rId14" xr:uid="{56EA8146-7375-2940-8CE7-621D3D82E155}"/>
-    <hyperlink ref="W15" r:id="rId15" xr:uid="{B991F48F-963A-5548-9E1D-97F06C683698}"/>
-    <hyperlink ref="W20" r:id="rId16" xr:uid="{AE74A4E6-305E-5F49-B0FE-9AAB97F6A3DF}"/>
-    <hyperlink ref="W40" r:id="rId17" xr:uid="{58E4C55D-2972-6044-88B9-E8D053273528}"/>
+    <hyperlink ref="X16" r:id="rId1" xr:uid="{06435D38-8656-894B-97C5-96B4F9A81B16}"/>
+    <hyperlink ref="X2" r:id="rId2" xr:uid="{EB14855D-0E7A-E441-A18B-4D016EB12E29}"/>
+    <hyperlink ref="X3" r:id="rId3" xr:uid="{C15DA009-4697-1244-8BAF-3240FF96A711}"/>
+    <hyperlink ref="X4" r:id="rId4" xr:uid="{5E45C078-1936-E646-A05B-0E269E699502}"/>
+    <hyperlink ref="X5" r:id="rId5" xr:uid="{3508BBD7-0686-214F-A732-F9D99867F37B}"/>
+    <hyperlink ref="X6" r:id="rId6" xr:uid="{44518A87-F14F-2046-B2D0-50BABBFE9F23}"/>
+    <hyperlink ref="X7" r:id="rId7" xr:uid="{9C71B0A9-7283-EE47-AD40-883AED7F6E3B}"/>
+    <hyperlink ref="X8" r:id="rId8" xr:uid="{A85AF766-CAB8-B745-B598-2A8703297230}"/>
+    <hyperlink ref="X9" r:id="rId9" xr:uid="{F4B0D80A-79B6-DA48-A301-0E18C15056FB}"/>
+    <hyperlink ref="X10" r:id="rId10" xr:uid="{3BA8B50E-BC9D-474A-B127-1A577C5A99E5}"/>
+    <hyperlink ref="X11" r:id="rId11" xr:uid="{D5D753E2-5C02-104F-8613-55614BC4ECCC}"/>
+    <hyperlink ref="X12" r:id="rId12" xr:uid="{F1B98F28-3440-4A4D-83F2-020B386BE961}"/>
+    <hyperlink ref="X13" r:id="rId13" xr:uid="{CEF4A8E3-B3D1-6D41-BC9D-129C9F04AB13}"/>
+    <hyperlink ref="X14" r:id="rId14" xr:uid="{7E56F984-036C-054B-AC54-65CDB8B27F35}"/>
+    <hyperlink ref="X15" r:id="rId15" xr:uid="{9464CCC8-2CFE-574E-A143-DA3F1F527DE6}"/>
+    <hyperlink ref="X20" r:id="rId16" xr:uid="{2FC3FD58-112F-F84B-9085-DE9B38C1019B}"/>
+    <hyperlink ref="X40" r:id="rId17" xr:uid="{DF8C6875-75B1-2349-8BCD-C0BD730420EB}"/>
+    <hyperlink ref="X39" r:id="rId18" xr:uid="{AC8170B0-D17B-354F-9989-7415944888AE}"/>
+    <hyperlink ref="X36" r:id="rId19" xr:uid="{CE12026F-61DF-C042-AA3B-3849F3B3051B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId18"/>
+  <legacyDrawing r:id="rId20"/>
   <tableParts count="1">
-    <tablePart r:id="rId19"/>
+    <tablePart r:id="rId21"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
actualizacion sal de oro II
</commit_message>
<xml_diff>
--- a/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
+++ b/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/rigi-dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFE43CF1-466E-8E47-B77C-8FF110ADE773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0085A19-ECED-6C4C-89CD-B1A7BE41161F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36440" yWindow="0" windowWidth="32360" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="1160" windowWidth="32360" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <author>tc={EA61046C-C94E-C449-8761-ABD505A37332}</author>
     <author>tc={9E845984-16BC-D640-8568-DCBC39BD282B}</author>
     <author>tc={D756854B-3370-2C47-8E59-D458EBCA5109}</author>
-    <author>tc={909B81E5-AB38-BB4F-A77E-C63D2711848A}</author>
+    <author>tc={F654CC8D-FD5A-6343-8A74-B7DC43C44B1A}</author>
   </authors>
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0" xr:uid="{CC7FC192-DD2F-524F-965B-B519233399BD}">
@@ -78,7 +78,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="N3" authorId="4" shapeId="0" xr:uid="{909B81E5-AB38-BB4F-A77E-C63D2711848A}">
+    <comment ref="N3" authorId="4" shapeId="0" xr:uid="{F654CC8D-FD5A-6343-8A74-B7DC43C44B1A}">
       <text>
         <t xml:space="preserve">[Comentario encadenado]
 Tu versión de Excel te permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="315">
   <si>
     <t>id_proyecto</t>
   </si>
@@ -442,13 +442,7 @@
     <t>Sucursal Dedicada Midstream RDA</t>
   </si>
   <si>
-    <t>Sal de Oro</t>
-  </si>
-  <si>
     <t>Posco (Corea del Sur)</t>
-  </si>
-  <si>
-    <t>Argentina S.A. (Posco)</t>
   </si>
   <si>
     <t>Sal de Vida</t>
@@ -1041,6 +1035,30 @@
   <si>
     <t>Extracción, producción y exportación de cobre, oro y plata de los yacimientos Josemaría y Filo del Sol ubicados en la provincia de San Juan, República Argentina, así como la exploración de las concesiones mineras que forman parte del proyecto y el desarrollo de la infraestructura necesaria para su ejecución. Incluye infraestructura clave para operaciones de minería a cielo abierto: una planta concentradora para el procesamiento de minerales, instalaciones de lixiviación, infraestructura eléctrica, sistemas de suministro de agua, caminos de acceso y alojamientos.</t>
   </si>
+  <si>
+    <t>Sal de Oro II</t>
+  </si>
+  <si>
+    <t>Construcción de una planta destinada a la producción de carbonato de litio y su infraestructura complementaria. La planta tendrá una capacidad operativa aproximada de 23.000 toneladas anuales, que se obtendrá a través de un proceso convencional de evaporación solar y tratamiento químico de salmuera.</t>
+  </si>
+  <si>
+    <t>Posco Argentina SAU SDE</t>
+  </si>
+  <si>
+    <t>30-71922048-3</t>
+  </si>
+  <si>
+    <t>Res. 1157/2026</t>
+  </si>
+  <si>
+    <t>Signos fuertes de preexistencia del Proyecto Sal de Oro II. POSCO Holdings aprobó la inversión de la segunda fase en octubre de 2022; en junio de 2023, antes del primer anuncio del RIGI, el Gobierno nacional y la empresa comunicaron el inicio de construcción de una planta de carbonato de litio de 23.000 toneladas anuales; y en abril de 2024 POSCO obtuvo financiamiento por hasta USD 668 millones para esa misma fase. Las coincidencias de empresa, localización, producto, capacidad y etapa indican que se trata sustancialmente del mismo proyecto incorporado posteriormente al régimen.</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/345279/20260731</t>
+  </si>
+  <si>
+    <t>Res. 1157/2026; Globaris; MECON</t>
+  </si>
 </sst>
 </file>
 
@@ -1049,7 +1067,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1107,23 +1125,10 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF212529"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1189,7 +1194,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1225,19 +1230,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1247,7 +1240,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Notas" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="28">
+  <dxfs count="27">
     <dxf>
       <font>
         <strike val="0"/>
@@ -1267,6 +1260,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
@@ -1293,7 +1287,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1554,7 +1548,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1641,20 +1635,6 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1722,7 +1702,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3BC5949B-99C1-C640-8DA2-C585B697BBE1}" name="ProyectosIntegrados2" displayName="ProyectosIntegrados2" ref="A1:Y40" headerRowDxfId="27" dataDxfId="26" totalsRowDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3BC5949B-99C1-C640-8DA2-C585B697BBE1}" name="ProyectosIntegrados2" displayName="ProyectosIntegrados2" ref="A1:Y40" headerRowDxfId="26" totalsRowDxfId="25">
   <tableColumns count="25">
     <tableColumn id="2" xr3:uid="{1FB8F74D-9682-B440-94D1-B6000493E00B}" name="VPU" dataDxfId="24"/>
     <tableColumn id="22" xr3:uid="{5F9EE6EB-2E4C-E743-B117-A1464438FFC7}" name="Descripción_del_proyecto" dataDxfId="23"/>
@@ -1747,7 +1727,7 @@
     <tableColumn id="15" xr3:uid="{AB9E3FD5-D9E1-FB4C-805E-4DC1E2E4F884}" name="norma_aprobacion" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{32A3F66C-F383-6A4F-BC9B-CE60E9775140}" name="Clasificacion_preexistencia_boletin_oficial" dataDxfId="3"/>
     <tableColumn id="23" xr3:uid="{8FFE7748-3D7D-F44F-9EE0-37998D10E3B7}" name="Justificacion_preexistencia_boletin_oficial" dataDxfId="2"/>
-    <tableColumn id="16" xr3:uid="{B5F0282B-C127-7C40-86CC-663CD39DAAF5}" name="link_norma" dataDxfId="1"/>
+    <tableColumn id="16" xr3:uid="{B5F0282B-C127-7C40-86CC-663CD39DAAF5}" name="link_norma" dataDxfId="1" dataCellStyle="Hipervínculo"/>
     <tableColumn id="20" xr3:uid="{4245686F-374C-B840-9963-4B9AF6D5BD62}" name="Fuentes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1945,7 +1925,7 @@
     <text xml:space="preserve">La fuente de datos de esta variable es el monitor del RIGI del MECON
 </text>
   </threadedComment>
-  <threadedComment ref="N3" dT="2026-06-09T13:10:11.61" personId="{2E8DF262-CB25-3049-80AF-0C6513AADFB8}" id="{909B81E5-AB38-BB4F-A77E-C63D2711848A}">
+  <threadedComment ref="N3" dT="2026-06-09T13:10:11.61" personId="{2E8DF262-CB25-3049-80AF-0C6513AADFB8}" id="{F654CC8D-FD5A-6343-8A74-B7DC43C44B1A}">
     <text xml:space="preserve">Que el solicitante declaró que el proyecto implicará una inversión total de entre dólares estadounidenses dos mil novecientos millones (USD 2.900.000.000) y dólares estadounidenses tres mil doscientos millones (USD 3.200.000.000). Se computa el promedio
 </text>
   </threadedComment>
@@ -1957,18 +1937,18 @@
   <dimension ref="A1:Y49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="94.33203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="16384" width="94.33203125" style="16"/>
+    <col min="1" max="16384" width="94.33203125" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
@@ -1977,10 +1957,10 @@
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>2</v>
@@ -1989,7 +1969,7 @@
         <v>3</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>4</v>
@@ -1998,43 +1978,43 @@
         <v>5</v>
       </c>
       <c r="M1" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="N1" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>148</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="R1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="U1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="X1" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="Y1" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.15">
@@ -2042,10 +2022,10 @@
         <v>40</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D2" s="8">
         <v>7</v>
@@ -2054,19 +2034,19 @@
         <v>41</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K2" s="7" t="s">
         <v>42</v>
@@ -2102,27 +2082,27 @@
         <v>43</v>
       </c>
       <c r="V2" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W2" s="7" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="X2" s="11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="Y2" s="7" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D3" s="8">
         <v>13</v>
@@ -2134,16 +2114,16 @@
         <v>67</v>
       </c>
       <c r="G3" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>175</v>
-      </c>
       <c r="J3" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>42</v>
@@ -2179,27 +2159,27 @@
         <v>68</v>
       </c>
       <c r="V3" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W3" s="7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="X3" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="Y3" s="7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A4" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D4" s="8">
         <v>33</v>
@@ -2211,7 +2191,7 @@
         <v>76</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>19</v>
@@ -2220,7 +2200,7 @@
         <v>52</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>25</v>
@@ -2256,27 +2236,27 @@
         <v>77</v>
       </c>
       <c r="V4" s="7" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="W4" s="7" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="Y4" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="60" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D5" s="8">
         <v>10</v>
@@ -2288,7 +2268,7 @@
         <v>55</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>19</v>
@@ -2297,7 +2277,7 @@
         <v>56</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>20</v>
@@ -2333,16 +2313,16 @@
         <v>57</v>
       </c>
       <c r="V5" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="W5" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="X5" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="Y5" s="7" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="45" x14ac:dyDescent="0.15">
@@ -2350,10 +2330,10 @@
         <v>49</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D6" s="8">
         <v>9</v>
@@ -2365,7 +2345,7 @@
         <v>51</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>19</v>
@@ -2374,7 +2354,7 @@
         <v>52</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>38</v>
@@ -2410,27 +2390,27 @@
         <v>53</v>
       </c>
       <c r="V6" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="X6" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D7" s="8">
         <v>3</v>
@@ -2442,16 +2422,16 @@
         <v>24</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>25</v>
@@ -2487,27 +2467,27 @@
         <v>27</v>
       </c>
       <c r="V7" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="W7" s="13" t="s">
-        <v>233</v>
+        <v>180</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>231</v>
       </c>
       <c r="X7" s="12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="Y7" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D8" s="8">
         <v>1</v>
@@ -2519,22 +2499,22 @@
         <v>9</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="M8" s="9">
         <v>550</v>
@@ -2564,27 +2544,27 @@
         <v>13</v>
       </c>
       <c r="V8" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="W8" s="7" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="X8" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="Y8" s="7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>291</v>
+      <c r="B9" s="7" t="s">
+        <v>289</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D9" s="8">
         <v>2</v>
@@ -2595,20 +2575,20 @@
       <c r="F9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="14" t="s">
-        <v>199</v>
+      <c r="G9" s="7" t="s">
+        <v>197</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>179</v>
+        <v>187</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>177</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>21</v>
@@ -2641,27 +2621,27 @@
         <v>22</v>
       </c>
       <c r="V9" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W9" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="X9" s="15" t="s">
-        <v>159</v>
+        <v>233</v>
+      </c>
+      <c r="X9" s="12" t="s">
+        <v>157</v>
       </c>
       <c r="Y9" s="7" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="75" x14ac:dyDescent="0.15">
-      <c r="A10" s="14" t="s">
-        <v>203</v>
+      <c r="A10" s="7" t="s">
+        <v>201</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D10" s="8">
         <v>14</v>
@@ -2670,19 +2650,19 @@
         <v>69</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>202</v>
+        <v>203</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>200</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="J10" s="14" t="s">
-        <v>204</v>
+        <v>187</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>202</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>25</v>
@@ -2717,17 +2697,17 @@
       <c r="U10" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="V10" s="14" t="s">
-        <v>169</v>
+      <c r="V10" s="7" t="s">
+        <v>167</v>
       </c>
       <c r="W10" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="X10" s="15" t="s">
-        <v>201</v>
+        <v>234</v>
+      </c>
+      <c r="X10" s="12" t="s">
+        <v>199</v>
       </c>
       <c r="Y10" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="75" x14ac:dyDescent="0.15">
@@ -2735,10 +2715,10 @@
         <v>44</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D11" s="8">
         <v>8</v>
@@ -2750,7 +2730,7 @@
         <v>46</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>47</v>
@@ -2759,7 +2739,7 @@
         <v>47</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>32</v>
@@ -2795,27 +2775,27 @@
         <v>48</v>
       </c>
       <c r="V11" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W11" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="X11" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="Y11" s="7" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:25" ht="60" x14ac:dyDescent="0.15">
       <c r="A12" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D12" s="8">
         <v>12</v>
@@ -2827,7 +2807,7 @@
         <v>61</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>62</v>
@@ -2836,7 +2816,7 @@
         <v>63</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>64</v>
@@ -2872,16 +2852,16 @@
         <v>65</v>
       </c>
       <c r="V12" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W12" s="7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="X12" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="Y12" s="7" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="120" x14ac:dyDescent="0.15">
@@ -2889,10 +2869,10 @@
         <v>28</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D13" s="8">
         <v>4</v>
@@ -2904,7 +2884,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>10</v>
@@ -2949,27 +2929,27 @@
         <v>34</v>
       </c>
       <c r="V13" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W13" s="7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="X13" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="Y13" s="7" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:25" ht="120" x14ac:dyDescent="0.15">
-      <c r="A14" s="17" t="s">
-        <v>306</v>
+      <c r="A14" s="7" t="s">
+        <v>304</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D14" s="8">
         <v>11</v>
@@ -2978,10 +2958,10 @@
         <v>54</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>19</v>
@@ -2990,7 +2970,7 @@
         <v>56</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>58</v>
@@ -3026,16 +3006,16 @@
         <v>59</v>
       </c>
       <c r="V14" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="W14" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="X14" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="45" x14ac:dyDescent="0.15">
@@ -3043,10 +3023,10 @@
         <v>71</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D15" s="8">
         <v>39</v>
@@ -3058,7 +3038,7 @@
         <v>73</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>19</v>
@@ -3067,7 +3047,7 @@
         <v>56</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>58</v>
@@ -3103,16 +3083,16 @@
         <v>74</v>
       </c>
       <c r="V15" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="W15" s="7" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="X15" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="Y15" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="45" x14ac:dyDescent="0.15">
@@ -3120,10 +3100,10 @@
         <v>35</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D16" s="8">
         <v>5</v>
@@ -3135,13 +3115,13 @@
         <v>37</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="J16" s="7"/>
       <c r="K16" s="7" t="s">
@@ -3178,16 +3158,16 @@
         <v>39</v>
       </c>
       <c r="V16" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="W16" s="13" t="s">
-        <v>242</v>
+        <v>180</v>
+      </c>
+      <c r="W16" s="7" t="s">
+        <v>240</v>
       </c>
       <c r="X16" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="Y16" s="7" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:25" ht="15" x14ac:dyDescent="0.15">
@@ -3227,7 +3207,7 @@
       </c>
       <c r="O17" s="9"/>
       <c r="P17" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q17" s="7"/>
       <c r="R17" s="10">
@@ -3240,14 +3220,14 @@
       <c r="W17" s="7"/>
       <c r="X17" s="12"/>
       <c r="Y17" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="18" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A18" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="14"/>
+      <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="8">
         <v>16</v>
@@ -3258,14 +3238,14 @@
       <c r="F18" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G18" s="14"/>
+      <c r="G18" s="7"/>
       <c r="H18" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="J18" s="14"/>
+      <c r="J18" s="7"/>
       <c r="K18" s="7" t="s">
         <v>85</v>
       </c>
@@ -3280,7 +3260,7 @@
       </c>
       <c r="O18" s="9"/>
       <c r="P18" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q18" s="7"/>
       <c r="R18" s="10">
@@ -3291,13 +3271,13 @@
       <c r="U18" s="7"/>
       <c r="V18" s="7"/>
       <c r="W18" s="7"/>
-      <c r="X18" s="15"/>
+      <c r="X18" s="12"/>
       <c r="Y18" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" spans="1:25" ht="15" x14ac:dyDescent="0.15">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="7" t="s">
         <v>86</v>
       </c>
       <c r="B19" s="7"/>
@@ -3311,14 +3291,14 @@
       <c r="F19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G19" s="14"/>
+      <c r="G19" s="7"/>
       <c r="H19" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J19" s="14"/>
+      <c r="J19" s="7"/>
       <c r="K19" s="7" t="s">
         <v>89</v>
       </c>
@@ -3333,7 +3313,7 @@
       </c>
       <c r="O19" s="9"/>
       <c r="P19" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q19" s="7"/>
       <c r="R19" s="10">
@@ -3344,20 +3324,20 @@
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
       <c r="W19" s="7"/>
-      <c r="X19" s="15"/>
+      <c r="X19" s="12"/>
       <c r="Y19" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="20" spans="1:25" ht="45" x14ac:dyDescent="0.15">
       <c r="A20" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>225</v>
+        <v>217</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>223</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D20" s="8">
         <v>18</v>
@@ -3366,10 +3346,10 @@
         <v>90</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>220</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>19</v>
@@ -3377,8 +3357,8 @@
       <c r="I20" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J20" s="14" t="s">
-        <v>220</v>
+      <c r="J20" s="7" t="s">
+        <v>218</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>91</v>
@@ -3411,26 +3391,26 @@
         <v>46177</v>
       </c>
       <c r="U20" s="7" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="V20" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="W20" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="X20" s="15" t="s">
-        <v>224</v>
+        <v>241</v>
+      </c>
+      <c r="X20" s="12" t="s">
+        <v>222</v>
       </c>
       <c r="Y20" s="7" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21" spans="1:25" ht="15" x14ac:dyDescent="0.15">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="14"/>
+      <c r="B21" s="7"/>
       <c r="C21" s="7"/>
       <c r="D21" s="8">
         <v>19</v>
@@ -3438,17 +3418,17 @@
       <c r="E21" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G21" s="14"/>
+      <c r="G21" s="7"/>
       <c r="H21" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J21" s="14"/>
+      <c r="J21" s="7"/>
       <c r="K21" s="7" t="s">
         <v>89</v>
       </c>
@@ -3463,7 +3443,7 @@
       </c>
       <c r="O21" s="9"/>
       <c r="P21" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q21" s="7"/>
       <c r="R21" s="10">
@@ -3474,9 +3454,9 @@
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
       <c r="W21" s="7"/>
-      <c r="X21" s="15"/>
+      <c r="X21" s="12"/>
       <c r="Y21" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:25" ht="15" x14ac:dyDescent="0.15">
@@ -3494,7 +3474,7 @@
       <c r="F22" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="G22" s="14"/>
+      <c r="G22" s="7"/>
       <c r="H22" s="9" t="s">
         <v>19</v>
       </c>
@@ -3516,7 +3496,7 @@
       </c>
       <c r="O22" s="9"/>
       <c r="P22" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q22" s="7"/>
       <c r="R22" s="10">
@@ -3527,13 +3507,13 @@
       <c r="U22" s="7"/>
       <c r="V22" s="7"/>
       <c r="W22" s="7"/>
-      <c r="X22" s="15"/>
+      <c r="X22" s="12"/>
       <c r="Y22" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" spans="1:25" ht="15" x14ac:dyDescent="0.15">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="7" t="s">
         <v>98</v>
       </c>
       <c r="B23" s="7"/>
@@ -3547,14 +3527,14 @@
       <c r="F23" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G23" s="14"/>
+      <c r="G23" s="7"/>
       <c r="H23" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J23" s="14"/>
+      <c r="J23" s="7"/>
       <c r="K23" s="7" t="s">
         <v>89</v>
       </c>
@@ -3569,7 +3549,7 @@
       </c>
       <c r="O23" s="9"/>
       <c r="P23" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q23" s="7"/>
       <c r="R23" s="10">
@@ -3580,16 +3560,16 @@
       <c r="U23" s="7"/>
       <c r="V23" s="7"/>
       <c r="W23" s="7"/>
-      <c r="X23" s="15"/>
+      <c r="X23" s="12"/>
       <c r="Y23" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="24" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A24" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="B24" s="14"/>
+        <v>134</v>
+      </c>
+      <c r="B24" s="7"/>
       <c r="C24" s="7"/>
       <c r="D24" s="8">
         <v>37</v>
@@ -3598,16 +3578,16 @@
         <v>114</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="G24" s="14"/>
+        <v>135</v>
+      </c>
+      <c r="G24" s="7"/>
       <c r="H24" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I24" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J24" s="14"/>
+      <c r="J24" s="7"/>
       <c r="K24" s="7" t="s">
         <v>32</v>
       </c>
@@ -3622,7 +3602,7 @@
       </c>
       <c r="O24" s="9"/>
       <c r="P24" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q24" s="7"/>
       <c r="R24" s="10">
@@ -3633,44 +3613,44 @@
       <c r="U24" s="7"/>
       <c r="V24" s="7"/>
       <c r="W24" s="7"/>
-      <c r="X24" s="15"/>
+      <c r="X24" s="12"/>
       <c r="Y24" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="25" spans="1:25" ht="90" x14ac:dyDescent="0.15">
       <c r="A25" s="7" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D25" s="8">
         <v>38</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="L25" s="7" t="s">
         <v>12</v>
@@ -3700,24 +3680,24 @@
         <v>46198</v>
       </c>
       <c r="U25" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="V25" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="W25" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="X25" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="Y25" s="7" t="s">
         <v>266</v>
-      </c>
-      <c r="V25" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="W25" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="X25" s="12" t="s">
-        <v>267</v>
-      </c>
-      <c r="Y25" s="7" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="26" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A26" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -3725,10 +3705,10 @@
         <v>40</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G26" s="7"/>
       <c r="H26" s="9" t="s">
@@ -3752,7 +3732,7 @@
       </c>
       <c r="O26" s="9"/>
       <c r="P26" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q26" s="7"/>
       <c r="R26" s="10">
@@ -3765,12 +3745,12 @@
       <c r="W26" s="7"/>
       <c r="X26" s="7"/>
       <c r="Y26" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="27" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A27" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -3778,7 +3758,7 @@
         <v>41</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>14</v>
@@ -3805,7 +3785,7 @@
       </c>
       <c r="O27" s="9"/>
       <c r="P27" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q27" s="7"/>
       <c r="R27" s="10">
@@ -3818,12 +3798,12 @@
       <c r="W27" s="7"/>
       <c r="X27" s="7"/>
       <c r="Y27" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="28" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A28" s="7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -3831,7 +3811,7 @@
         <v>32</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>14</v>
@@ -3858,7 +3838,7 @@
       </c>
       <c r="O28" s="9"/>
       <c r="P28" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q28" s="7"/>
       <c r="R28" s="10">
@@ -3871,32 +3851,32 @@
       <c r="W28" s="7"/>
       <c r="X28" s="7"/>
       <c r="Y28" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="29" spans="1:25" ht="15" x14ac:dyDescent="0.15">
-      <c r="A29" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="B29" s="14"/>
+      <c r="A29" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="8">
         <v>34</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="G29" s="14"/>
+        <v>127</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="G29" s="7"/>
       <c r="H29" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J29" s="14"/>
+      <c r="J29" s="7"/>
       <c r="K29" s="7" t="s">
         <v>20</v>
       </c>
@@ -3911,7 +3891,7 @@
       </c>
       <c r="O29" s="9"/>
       <c r="P29" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="Q29" s="7"/>
       <c r="R29" s="10">
@@ -3924,12 +3904,12 @@
       <c r="W29" s="7"/>
       <c r="X29" s="7"/>
       <c r="Y29" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="30" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A30" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -3937,10 +3917,10 @@
         <v>35</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G30" s="7"/>
       <c r="H30" s="9" t="s">
@@ -3964,7 +3944,7 @@
       </c>
       <c r="O30" s="9"/>
       <c r="P30" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q30" s="7"/>
       <c r="R30" s="10">
@@ -3977,12 +3957,12 @@
       <c r="W30" s="7"/>
       <c r="X30" s="7"/>
       <c r="Y30" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A31" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -3993,7 +3973,7 @@
         <v>96</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G31" s="7"/>
       <c r="H31" s="9" t="s">
@@ -4017,7 +3997,7 @@
       </c>
       <c r="O31" s="9"/>
       <c r="P31" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q31" s="7"/>
       <c r="R31" s="10">
@@ -4030,7 +4010,7 @@
       <c r="W31" s="7"/>
       <c r="X31" s="7"/>
       <c r="Y31" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:25" ht="15" x14ac:dyDescent="0.15">
@@ -4070,7 +4050,7 @@
       </c>
       <c r="O32" s="9"/>
       <c r="P32" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q32" s="7"/>
       <c r="R32" s="10" t="s">
@@ -4083,7 +4063,7 @@
       <c r="W32" s="7"/>
       <c r="X32" s="7"/>
       <c r="Y32" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" spans="1:25" ht="15" x14ac:dyDescent="0.15">
@@ -4123,7 +4103,7 @@
       </c>
       <c r="O33" s="9"/>
       <c r="P33" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q33" s="7"/>
       <c r="R33" s="10">
@@ -4136,7 +4116,7 @@
       <c r="W33" s="7"/>
       <c r="X33" s="7"/>
       <c r="Y33" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="34" spans="1:25" ht="15" x14ac:dyDescent="0.15">
@@ -4176,7 +4156,7 @@
       </c>
       <c r="O34" s="9"/>
       <c r="P34" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q34" s="7"/>
       <c r="R34" s="10">
@@ -4189,7 +4169,7 @@
       <c r="W34" s="7"/>
       <c r="X34" s="7"/>
       <c r="Y34" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="35" spans="1:25" ht="15" x14ac:dyDescent="0.15">
@@ -4229,7 +4209,7 @@
       </c>
       <c r="O35" s="9"/>
       <c r="P35" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q35" s="7"/>
       <c r="R35" s="10">
@@ -4242,18 +4222,18 @@
       <c r="W35" s="7"/>
       <c r="X35" s="7"/>
       <c r="Y35" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="36" spans="1:25" ht="90" x14ac:dyDescent="0.15">
       <c r="A36" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="B36" s="17" t="s">
-        <v>275</v>
+        <v>268</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>273</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D36" s="8">
         <v>26</v>
@@ -4264,17 +4244,17 @@
       <c r="F36" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="G36" s="17" t="s">
-        <v>274</v>
+      <c r="G36" s="7" t="s">
+        <v>272</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="J36" s="17" t="s">
-        <v>273</v>
+        <v>163</v>
+      </c>
+      <c r="J36" s="7" t="s">
+        <v>271</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>89</v>
@@ -4307,77 +4287,101 @@
         <v>46224</v>
       </c>
       <c r="U36" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="V36" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="W36" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="X36" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y36" s="7" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25" ht="90" x14ac:dyDescent="0.15">
+      <c r="A37" s="7" t="s">
         <v>307</v>
       </c>
-      <c r="V36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="W36" s="16" t="s">
-        <v>276</v>
-      </c>
-      <c r="X36" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="Y36" s="7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="37" spans="1:25" ht="15" x14ac:dyDescent="0.15">
-      <c r="A37" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
+      <c r="B37" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>180</v>
+      </c>
       <c r="D37" s="8">
         <v>27</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="G37" s="7"/>
+        <v>309</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>310</v>
+      </c>
       <c r="H37" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I37" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J37" s="7"/>
+      <c r="J37" s="7" t="s">
+        <v>184</v>
+      </c>
       <c r="K37" s="7" t="s">
-        <v>20</v>
+        <v>198</v>
       </c>
       <c r="L37" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M37" s="9">
-        <v>845</v>
+        <v>547</v>
       </c>
       <c r="N37" s="9">
-        <v>845</v>
-      </c>
-      <c r="O37" s="9"/>
+        <v>547</v>
+      </c>
+      <c r="O37" s="9">
+        <v>207.9364272</v>
+      </c>
       <c r="P37" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="Q37" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="Q37" s="7">
+        <v>2335</v>
+      </c>
       <c r="R37" s="10">
         <v>45595</v>
       </c>
-      <c r="S37" s="10"/>
-      <c r="T37" s="10"/>
-      <c r="U37" s="7"/>
-      <c r="V37" s="7"/>
-      <c r="W37" s="7"/>
-      <c r="X37" s="7"/>
+      <c r="S37" s="10">
+        <v>46185</v>
+      </c>
+      <c r="T37" s="10">
+        <v>46234</v>
+      </c>
+      <c r="U37" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="V37" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="W37" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="X37" s="7" t="s">
+        <v>313</v>
+      </c>
       <c r="Y37" s="7" t="s">
-        <v>226</v>
+        <v>314</v>
       </c>
     </row>
     <row r="38" spans="1:25" ht="15" x14ac:dyDescent="0.15">
       <c r="A38" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -4388,7 +4392,7 @@
         <v>54</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G38" s="7"/>
       <c r="H38" s="9" t="s">
@@ -4412,7 +4416,7 @@
       </c>
       <c r="O38" s="9"/>
       <c r="P38" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q38" s="7"/>
       <c r="R38" s="10">
@@ -4425,28 +4429,28 @@
       <c r="W38" s="7"/>
       <c r="X38" s="7"/>
       <c r="Y38" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" spans="1:25" ht="90" x14ac:dyDescent="0.15">
-      <c r="A39" s="17" t="s">
+      <c r="A39" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B39" s="7" t="s">
         <v>282</v>
-      </c>
-      <c r="B39" s="17" t="s">
-        <v>284</v>
       </c>
       <c r="C39" s="7"/>
       <c r="D39" s="8">
         <v>29</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="G39" s="17" t="s">
-        <v>281</v>
+        <v>120</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>279</v>
       </c>
       <c r="H39" s="9" t="s">
         <v>19</v>
@@ -4455,7 +4459,7 @@
         <v>56</v>
       </c>
       <c r="J39" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K39" s="7" t="s">
         <v>58</v>
@@ -4488,51 +4492,51 @@
         <v>46232</v>
       </c>
       <c r="U39" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="V39" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="W39" s="16" t="s">
-        <v>283</v>
-      </c>
-      <c r="X39" s="15" t="s">
-        <v>279</v>
+        <v>167</v>
+      </c>
+      <c r="W39" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="X39" s="12" t="s">
+        <v>277</v>
       </c>
       <c r="Y39" s="7" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="40" spans="1:25" ht="90" x14ac:dyDescent="0.15">
-      <c r="A40" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="B40" s="17" t="s">
-        <v>308</v>
+      <c r="A40" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>306</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D40" s="8">
         <v>31</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="G40" s="17" t="s">
-        <v>299</v>
+        <v>123</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>297</v>
       </c>
       <c r="H40" s="9" t="s">
         <v>19</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="J40" s="14" t="s">
-        <v>179</v>
+        <v>298</v>
+      </c>
+      <c r="J40" s="7" t="s">
+        <v>177</v>
       </c>
       <c r="K40" s="7" t="s">
         <v>25</v>
@@ -4565,19 +4569,19 @@
         <v>46233</v>
       </c>
       <c r="U40" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="V40" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="W40" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="X40" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="Y40" s="7" t="s">
         <v>301</v>
-      </c>
-      <c r="V40" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="W40" s="16" t="s">
-        <v>304</v>
-      </c>
-      <c r="X40" s="15" t="s">
-        <v>302</v>
-      </c>
-      <c r="Y40" s="7" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.15">
@@ -4817,25 +4821,25 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="X16" r:id="rId1" xr:uid="{06435D38-8656-894B-97C5-96B4F9A81B16}"/>
-    <hyperlink ref="X2" r:id="rId2" xr:uid="{EB14855D-0E7A-E441-A18B-4D016EB12E29}"/>
-    <hyperlink ref="X3" r:id="rId3" xr:uid="{C15DA009-4697-1244-8BAF-3240FF96A711}"/>
-    <hyperlink ref="X4" r:id="rId4" xr:uid="{5E45C078-1936-E646-A05B-0E269E699502}"/>
-    <hyperlink ref="X5" r:id="rId5" xr:uid="{3508BBD7-0686-214F-A732-F9D99867F37B}"/>
-    <hyperlink ref="X6" r:id="rId6" xr:uid="{44518A87-F14F-2046-B2D0-50BABBFE9F23}"/>
-    <hyperlink ref="X7" r:id="rId7" xr:uid="{9C71B0A9-7283-EE47-AD40-883AED7F6E3B}"/>
-    <hyperlink ref="X8" r:id="rId8" xr:uid="{A85AF766-CAB8-B745-B598-2A8703297230}"/>
-    <hyperlink ref="X9" r:id="rId9" xr:uid="{F4B0D80A-79B6-DA48-A301-0E18C15056FB}"/>
-    <hyperlink ref="X10" r:id="rId10" xr:uid="{3BA8B50E-BC9D-474A-B127-1A577C5A99E5}"/>
-    <hyperlink ref="X11" r:id="rId11" xr:uid="{D5D753E2-5C02-104F-8613-55614BC4ECCC}"/>
-    <hyperlink ref="X12" r:id="rId12" xr:uid="{F1B98F28-3440-4A4D-83F2-020B386BE961}"/>
-    <hyperlink ref="X13" r:id="rId13" xr:uid="{CEF4A8E3-B3D1-6D41-BC9D-129C9F04AB13}"/>
-    <hyperlink ref="X14" r:id="rId14" xr:uid="{7E56F984-036C-054B-AC54-65CDB8B27F35}"/>
-    <hyperlink ref="X15" r:id="rId15" xr:uid="{9464CCC8-2CFE-574E-A143-DA3F1F527DE6}"/>
-    <hyperlink ref="X20" r:id="rId16" xr:uid="{2FC3FD58-112F-F84B-9085-DE9B38C1019B}"/>
-    <hyperlink ref="X40" r:id="rId17" xr:uid="{DF8C6875-75B1-2349-8BCD-C0BD730420EB}"/>
-    <hyperlink ref="X39" r:id="rId18" xr:uid="{AC8170B0-D17B-354F-9989-7415944888AE}"/>
-    <hyperlink ref="X36" r:id="rId19" xr:uid="{CE12026F-61DF-C042-AA3B-3849F3B3051B}"/>
+    <hyperlink ref="X16" r:id="rId1" xr:uid="{D2412230-C3CD-7141-A25E-81BAF21A6174}"/>
+    <hyperlink ref="X2" r:id="rId2" xr:uid="{6D3504F9-33D3-5C42-ADC4-1F1B36F66242}"/>
+    <hyperlink ref="X3" r:id="rId3" xr:uid="{46673F91-F8F5-E946-A08B-B67632A08D9A}"/>
+    <hyperlink ref="X4" r:id="rId4" xr:uid="{68D4EB52-1EA3-C340-8AD8-D38DE0C9F22E}"/>
+    <hyperlink ref="X5" r:id="rId5" xr:uid="{012259F1-B4A3-1045-9E7A-AA126AE86681}"/>
+    <hyperlink ref="X6" r:id="rId6" xr:uid="{2C8B22AB-5777-4540-9E80-66B0C685703B}"/>
+    <hyperlink ref="X7" r:id="rId7" xr:uid="{49A07586-1F8E-8B41-AEA7-4C3E0536DD20}"/>
+    <hyperlink ref="X8" r:id="rId8" xr:uid="{56C3B5AD-00FB-E64B-9608-926539AA5FD6}"/>
+    <hyperlink ref="X9" r:id="rId9" xr:uid="{55AFF93D-C6FF-614A-B18E-808BD1FB3040}"/>
+    <hyperlink ref="X10" r:id="rId10" xr:uid="{4C306BC4-9928-3645-BF72-CEF21D95B062}"/>
+    <hyperlink ref="X11" r:id="rId11" xr:uid="{E51E5B00-AE31-004C-80CA-1046BF32CCCF}"/>
+    <hyperlink ref="X12" r:id="rId12" xr:uid="{10235633-5E5E-DD47-9890-13CA8ADBFF10}"/>
+    <hyperlink ref="X13" r:id="rId13" xr:uid="{C5CA1D0E-3350-CC43-8953-1CB241BB051B}"/>
+    <hyperlink ref="X14" r:id="rId14" xr:uid="{51CBFD06-0CB5-2C42-8727-D4B9CB369184}"/>
+    <hyperlink ref="X15" r:id="rId15" xr:uid="{8F2DFA35-F36C-F944-9C1B-42BE62E36FAC}"/>
+    <hyperlink ref="X20" r:id="rId16" xr:uid="{6349A6AC-03EB-6D4A-8F5A-A51D3A9078D4}"/>
+    <hyperlink ref="X40" r:id="rId17" xr:uid="{32F573A4-ED90-7044-AEEE-F5401A638E68}"/>
+    <hyperlink ref="X39" r:id="rId18" xr:uid="{18E22821-D2A5-A440-B5C5-EDB3995DD45E}"/>
+    <hyperlink ref="X36" r:id="rId19" xr:uid="{027F49BC-6705-E14A-ACC3-B787972340B2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId20"/>
@@ -4855,7 +4859,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>